<commit_message>
Headers for the requested variables without one; commented varsets with all the pressure levels
- 57 headers (CORDEX-CMIP6, FPS-URB-RCC, FPS-LUCAS variables not yet
  written): metadata from the CORDEX-CMIP6 CMOR tables or the data
  requests, wrfvar the main WRF field, first line = the fields needed
  and 'no CORDEX_Cmor program yet'
- 20 and 10 hPa headers (ua, va, ta, hus, zg, wa) for the RCM_plev_*
  programs; the plev varsets with all the CORDEX-CMIP6 levels are added,
  commented, under the active ones in the three varset files
- CORDEX_Cmor_variables.csv/xlsx: 'header ready' in the comment;
  mrroLut fields as mrro (RUNSF RUNSB); README

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QusijEwmX4bwsbKvYikBaV
</commit_message>
<xml_diff>
--- a/CORDEX_Cmor_variables.xlsx
+++ b/CORDEX_Cmor_variables.xlsx
@@ -2012,7 +2012,7 @@
       </c>
       <c r="N25" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; daily maximum of the hourly precipitation</t>
+          <t>not produced by CORDEX_Cmor; header ready; daily maximum of the hourly precipitation</t>
         </is>
       </c>
     </row>
@@ -4004,7 +4004,7 @@
       </c>
       <c r="N56" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; vertical integral</t>
+          <t>not produced by CORDEX_Cmor; header ready; vertical integral</t>
         </is>
       </c>
     </row>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="N57" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; vertical integral (2-moment microphysics with hail)</t>
+          <t>not produced by CORDEX_Cmor; header ready; vertical integral (2-moment microphysics with hail)</t>
         </is>
       </c>
     </row>
@@ -8780,7 +8780,7 @@
       </c>
       <c r="N127" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; no gust diagnostic in the WRF output</t>
+          <t>not produced by CORDEX_Cmor; header ready; no gust diagnostic in the WRF output</t>
         </is>
       </c>
     </row>
@@ -9480,7 +9480,7 @@
       </c>
       <c r="N138" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; derived (e.g. wrf-python cape_2d)</t>
+          <t>not produced by CORDEX_Cmor; header ready; derived (e.g. wrf-python cape_2d)</t>
         </is>
       </c>
     </row>
@@ -9544,7 +9544,7 @@
       </c>
       <c r="N139" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; derived (lifted index at 500 hPa)</t>
+          <t>not produced by CORDEX_Cmor; header ready; derived (lifted index at 500 hPa)</t>
         </is>
       </c>
     </row>
@@ -9608,7 +9608,7 @@
       </c>
       <c r="N140" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; derived (e.g. wrf-python cape_2d)</t>
+          <t>not produced by CORDEX_Cmor; header ready; derived (e.g. wrf-python cape_2d)</t>
         </is>
       </c>
     </row>
@@ -9664,7 +9664,7 @@
       </c>
       <c r="N141" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; daily maximum of cape</t>
+          <t>not produced by CORDEX_Cmor; header ready; daily maximum of cape</t>
         </is>
       </c>
     </row>
@@ -9720,7 +9720,7 @@
       </c>
       <c r="N142" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; daily maximum of li</t>
+          <t>not produced by CORDEX_Cmor; header ready; daily maximum of li</t>
         </is>
       </c>
     </row>
@@ -9776,7 +9776,7 @@
       </c>
       <c r="N143" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; daily maximum of cin</t>
+          <t>not produced by CORDEX_Cmor; header ready; daily maximum of cin</t>
         </is>
       </c>
     </row>
@@ -10236,7 +10236,7 @@
       </c>
       <c r="N150" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor</t>
+          <t>not produced by CORDEX_Cmor; header ready; commented lines with all the pressure levels in config/varsets*.sh; missing unless p_top &lt; 20 hPa</t>
         </is>
       </c>
     </row>
@@ -10304,7 +10304,7 @@
       </c>
       <c r="N151" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; above the model top with p_top = 2000 Pa</t>
+          <t>not produced by CORDEX_Cmor; header ready; commented lines with all the pressure levels in config/varsets*.sh; missing unless p_top &lt; 10 hPa</t>
         </is>
       </c>
     </row>
@@ -10712,7 +10712,7 @@
       </c>
       <c r="N157" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor</t>
+          <t>not produced by CORDEX_Cmor; header ready; commented lines with all the pressure levels in config/varsets*.sh; missing unless p_top &lt; 20 hPa</t>
         </is>
       </c>
     </row>
@@ -10780,7 +10780,7 @@
       </c>
       <c r="N158" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; above the model top with p_top = 2000 Pa</t>
+          <t>not produced by CORDEX_Cmor; header ready; commented lines with all the pressure levels in config/varsets*.sh; missing unless p_top &lt; 10 hPa</t>
         </is>
       </c>
     </row>
@@ -11188,7 +11188,7 @@
       </c>
       <c r="N164" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor</t>
+          <t>not produced by CORDEX_Cmor; header ready; commented lines with all the pressure levels in config/varsets*.sh; missing unless p_top &lt; 20 hPa</t>
         </is>
       </c>
     </row>
@@ -11256,7 +11256,7 @@
       </c>
       <c r="N165" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; above the model top with p_top = 2000 Pa</t>
+          <t>not produced by CORDEX_Cmor; header ready; commented lines with all the pressure levels in config/varsets*.sh; missing unless p_top &lt; 10 hPa</t>
         </is>
       </c>
     </row>
@@ -11664,7 +11664,7 @@
       </c>
       <c r="N171" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor</t>
+          <t>not produced by CORDEX_Cmor; header ready; commented lines with all the pressure levels in config/varsets*.sh; missing unless p_top &lt; 20 hPa</t>
         </is>
       </c>
     </row>
@@ -11732,7 +11732,7 @@
       </c>
       <c r="N172" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; above the model top with p_top = 2000 Pa</t>
+          <t>not produced by CORDEX_Cmor; header ready; commented lines with all the pressure levels in config/varsets*.sh; missing unless p_top &lt; 10 hPa</t>
         </is>
       </c>
     </row>
@@ -12140,7 +12140,7 @@
       </c>
       <c r="N178" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor</t>
+          <t>not produced by CORDEX_Cmor; header ready; commented lines with all the pressure levels in config/varsets*.sh; missing unless p_top &lt; 20 hPa</t>
         </is>
       </c>
     </row>
@@ -12208,7 +12208,7 @@
       </c>
       <c r="N179" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; above the model top with p_top = 2000 Pa</t>
+          <t>not produced by CORDEX_Cmor; header ready; commented lines with all the pressure levels in config/varsets*.sh; missing unless p_top &lt; 10 hPa</t>
         </is>
       </c>
     </row>
@@ -12616,7 +12616,7 @@
       </c>
       <c r="N185" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor</t>
+          <t>not produced by CORDEX_Cmor; header ready; commented lines with all the pressure levels in config/varsets*.sh; missing unless p_top &lt; 20 hPa</t>
         </is>
       </c>
     </row>
@@ -12684,7 +12684,7 @@
       </c>
       <c r="N186" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; above the model top with p_top = 2000 Pa</t>
+          <t>not produced by CORDEX_Cmor; header ready; commented lines with all the pressure levels in config/varsets*.sh; missing unless p_top &lt; 10 hPa</t>
         </is>
       </c>
     </row>
@@ -13428,7 +13428,7 @@
       </c>
       <c r="N198" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; root layers per vegetation class (NROOT of VEGPARM.TBL)</t>
+          <t>not produced by CORDEX_Cmor; header ready; root layers per vegetation class (NROOT of VEGPARM.TBL)</t>
         </is>
       </c>
     </row>
@@ -13572,7 +13572,7 @@
       </c>
       <c r="N201" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; not available from WRF (external dataset)</t>
+          <t>not produced by CORDEX_Cmor; header ready; not available from WRF (external dataset)</t>
         </is>
       </c>
     </row>
@@ -13620,7 +13620,7 @@
       </c>
       <c r="N202" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; geo_em; DX*DY/(MAPFAC_MX*MAPFAC_MY) with the DX/DY attributes</t>
+          <t>not produced by CORDEX_Cmor; header ready; geo_em; DX*DY/(MAPFAC_MX*MAPFAC_MY) with the DX/DY attributes</t>
         </is>
       </c>
     </row>
@@ -13684,7 +13684,7 @@
       </c>
       <c r="N203" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor</t>
+          <t>not produced by CORDEX_Cmor; header ready</t>
         </is>
       </c>
     </row>
@@ -14000,7 +14000,7 @@
       </c>
       <c r="N208" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; not in the WRF history output</t>
+          <t>not produced by CORDEX_Cmor; header ready; not in the WRF history output</t>
         </is>
       </c>
     </row>
@@ -14624,7 +14624,7 @@
       </c>
       <c r="N218" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; geo_em; DX*DY/(MAPFAC_MX*MAPFAC_MY) with the DX/DY attributes</t>
+          <t>not produced by CORDEX_Cmor; header ready; geo_em; DX*DY/(MAPFAC_MX*MAPFAC_MY) with the DX/DY attributes</t>
         </is>
       </c>
     </row>
@@ -15072,7 +15072,7 @@
       </c>
       <c r="N226" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; model levels</t>
+          <t>not produced by CORDEX_Cmor; header ready; model levels</t>
         </is>
       </c>
     </row>
@@ -17900,7 +17900,7 @@
       </c>
       <c r="N277" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; no canopy albedo in the WRF output</t>
+          <t>not produced by CORDEX_Cmor; header ready; no canopy albedo in the WRF output</t>
         </is>
       </c>
     </row>
@@ -18100,7 +18100,7 @@
       </c>
       <c r="N281" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; Noah-MP with dynamic vegetation (opt_dveg)</t>
+          <t>not produced by CORDEX_Cmor; header ready; Noah-MP with dynamic vegetation (opt_dveg)</t>
         </is>
       </c>
     </row>
@@ -18316,7 +18316,7 @@
       </c>
       <c r="N285" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; no land-use tiles in WRF: grid-cell value only</t>
+          <t>not produced by CORDEX_Cmor; header ready; no land-use tiles in WRF: grid-cell value only</t>
         </is>
       </c>
     </row>
@@ -18372,7 +18372,7 @@
       </c>
       <c r="N286" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; no land-use tiles in WRF: grid-cell value only</t>
+          <t>not produced by CORDEX_Cmor; header ready; no land-use tiles in WRF: grid-cell value only</t>
         </is>
       </c>
     </row>
@@ -18428,7 +18428,7 @@
       </c>
       <c r="N287" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; no land-use tiles in WRF (Noah-MP Q2MV/Q2MB: vegetated/bare parts)</t>
+          <t>not produced by CORDEX_Cmor; header ready; no land-use tiles in WRF (Noah-MP Q2MV/Q2MB: vegetated/bare parts)</t>
         </is>
       </c>
     </row>
@@ -18484,7 +18484,7 @@
       </c>
       <c r="N288" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; Noah-MP canopy water</t>
+          <t>not produced by CORDEX_Cmor; header ready; Noah-MP canopy water</t>
         </is>
       </c>
     </row>
@@ -18540,7 +18540,7 @@
       </c>
       <c r="N289" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; Noah-MP irrigation (opt_irr); no land-use tiles</t>
+          <t>not produced by CORDEX_Cmor; header ready; Noah-MP irrigation (opt_irr); no land-use tiles</t>
         </is>
       </c>
     </row>
@@ -18596,7 +18596,7 @@
       </c>
       <c r="N290" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; no land-use tiles in WRF: grid-cell value only</t>
+          <t>not produced by CORDEX_Cmor; header ready; no land-use tiles in WRF: grid-cell value only</t>
         </is>
       </c>
     </row>
@@ -18644,7 +18644,7 @@
       </c>
       <c r="N291" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; one value per land-use class (needs a 3-D fx writer)</t>
+          <t>not produced by CORDEX_Cmor; header ready; one value per land-use class (needs a 3-D fx writer)</t>
         </is>
       </c>
     </row>
@@ -18695,12 +18695,12 @@
       </c>
       <c r="M292" s="4" t="inlineStr">
         <is>
-          <t>SFROFF UDROFF</t>
+          <t>RUNSF RUNSB</t>
         </is>
       </c>
       <c r="N292" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; no land-use tiles in WRF: grid-cell value only</t>
+          <t>not produced by CORDEX_Cmor; header ready; no land-use tiles in WRF: grid-cell value only</t>
         </is>
       </c>
     </row>
@@ -18756,7 +18756,7 @@
       </c>
       <c r="N293" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; no land-use tiles in WRF: grid-cell value only</t>
+          <t>not produced by CORDEX_Cmor; header ready; no land-use tiles in WRF: grid-cell value only</t>
         </is>
       </c>
     </row>
@@ -18812,7 +18812,7 @@
       </c>
       <c r="N294" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; no land-use tiles in WRF: grid-cell value only</t>
+          <t>not produced by CORDEX_Cmor; header ready; no land-use tiles in WRF: grid-cell value only</t>
         </is>
       </c>
     </row>
@@ -18868,7 +18868,7 @@
       </c>
       <c r="N295" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; Noah-MP with dynamic vegetation (opt_dveg)</t>
+          <t>not produced by CORDEX_Cmor; header ready; Noah-MP with dynamic vegetation (opt_dveg)</t>
         </is>
       </c>
     </row>
@@ -18916,7 +18916,7 @@
       </c>
       <c r="N296" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; no pasture class in the WRF land-use tables</t>
+          <t>not produced by CORDEX_Cmor; header ready; no pasture class in the WRF land-use tables</t>
         </is>
       </c>
     </row>
@@ -18964,7 +18964,7 @@
       </c>
       <c r="N297" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; urban + land ice classes; LUCAS name resdiualFrac</t>
+          <t>not produced by CORDEX_Cmor; header ready; urban + land ice classes; LUCAS name resdiualFrac</t>
         </is>
       </c>
     </row>
@@ -19020,7 +19020,7 @@
       </c>
       <c r="N298" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; no land-use tiles in WRF: grid-cell value only</t>
+          <t>not produced by CORDEX_Cmor; header ready; no land-use tiles in WRF: grid-cell value only</t>
         </is>
       </c>
     </row>
@@ -19076,7 +19076,7 @@
       </c>
       <c r="N299" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor</t>
+          <t>not produced by CORDEX_Cmor; header ready</t>
         </is>
       </c>
     </row>
@@ -19132,7 +19132,7 @@
       </c>
       <c r="N300" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; no land-use tiles in WRF: grid-cell value only</t>
+          <t>not produced by CORDEX_Cmor; header ready; no land-use tiles in WRF: grid-cell value only</t>
         </is>
       </c>
     </row>
@@ -19236,7 +19236,7 @@
       </c>
       <c r="N302" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; SNOW/1000; no land-use tiles in WRF</t>
+          <t>not produced by CORDEX_Cmor; header ready; SNOW/1000; no land-use tiles in WRF</t>
         </is>
       </c>
     </row>
@@ -19292,7 +19292,7 @@
       </c>
       <c r="N303" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; no land-use tiles in WRF (Noah-MP T2MV/T2MB: vegetated/bare parts)</t>
+          <t>not produced by CORDEX_Cmor; header ready; no land-use tiles in WRF (Noah-MP T2MV/T2MB: vegetated/bare parts)</t>
         </is>
       </c>
     </row>
@@ -19348,7 +19348,7 @@
       </c>
       <c r="N304" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; Noah-MP vegetation temperature</t>
+          <t>not produced by CORDEX_Cmor; header ready; Noah-MP vegetation temperature</t>
         </is>
       </c>
     </row>
@@ -19404,7 +19404,7 @@
       </c>
       <c r="N305" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; Noah-MP bare ground temperature</t>
+          <t>not produced by CORDEX_Cmor; header ready; Noah-MP bare ground temperature</t>
         </is>
       </c>
     </row>
@@ -19556,7 +19556,7 @@
       </c>
       <c r="N308" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; MODIS class 4 (deciduous broadleaf forest)</t>
+          <t>not produced by CORDEX_Cmor; header ready; MODIS class 4 (deciduous broadleaf forest)</t>
         </is>
       </c>
     </row>
@@ -19604,7 +19604,7 @@
       </c>
       <c r="N309" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; MODIS class 2 (evergreen broadleaf forest)</t>
+          <t>not produced by CORDEX_Cmor; header ready; MODIS class 2 (evergreen broadleaf forest)</t>
         </is>
       </c>
     </row>
@@ -19652,7 +19652,7 @@
       </c>
       <c r="N310" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; MODIS class 3 (deciduous needleleaf forest)</t>
+          <t>not produced by CORDEX_Cmor; header ready; MODIS class 3 (deciduous needleleaf forest)</t>
         </is>
       </c>
     </row>
@@ -19764,7 +19764,7 @@
       </c>
       <c r="N312" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; no land-use tiles in WRF: grid-cell value only</t>
+          <t>not produced by CORDEX_Cmor; header ready; no land-use tiles in WRF: grid-cell value only</t>
         </is>
       </c>
     </row>
@@ -19868,7 +19868,7 @@
       </c>
       <c r="N314" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; derived (e.g. wrf-python cape_2d); LUCAS name CAPE</t>
+          <t>not produced by CORDEX_Cmor; header ready; derived (e.g. wrf-python cape_2d); LUCAS name CAPE</t>
         </is>
       </c>
     </row>
@@ -19924,7 +19924,7 @@
       </c>
       <c r="N315" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; derived (e.g. wrf-python cape_2d); LUCAS name CIN</t>
+          <t>not produced by CORDEX_Cmor; header ready; derived (e.g. wrf-python cape_2d); LUCAS name CIN</t>
         </is>
       </c>
     </row>
@@ -19980,7 +19980,7 @@
       </c>
       <c r="N316" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; relative vorticity on pressure levels</t>
+          <t>not produced by CORDEX_Cmor; header ready; relative vorticity on pressure levels</t>
         </is>
       </c>
     </row>
@@ -20036,7 +20036,7 @@
       </c>
       <c r="N317" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; omega = -rho g w on pressure levels</t>
+          <t>not produced by CORDEX_Cmor; header ready; omega = -rho g w on pressure levels</t>
         </is>
       </c>
     </row>
@@ -20084,7 +20084,7 @@
       </c>
       <c r="N318" s="4" t="inlineStr">
         <is>
-          <t>not produced by CORDEX_Cmor; Noah-MP soil layer thickness</t>
+          <t>not produced by CORDEX_Cmor; header ready; Noah-MP soil layer thickness</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Omega on pressure levels: RCM_plev_wap, headers wap1000..wap10, plev_wap varset
- RCM_plev_wap.f90 (from the old RCM_50km_pl_omega): omega = -rho g w on
  the model levels (W averaged to the mass levels, T from theta', Tv with
  QVAPOR, p = P + PB), interpolated in log(p) to pres as RCM_plev_wa;
  every 6 h (wp_step); loops kept inside the model levels
- one header per pressure level (wap1000 ... wap30, wap20, wap10);
  header_wap (single, with the old 'set pres' note) removed
- plev_wap varset (self-looping, not in ORDER, 36 h) in the three varset
  files, with the commented line for all the levels
- variable list: wap written by RCM_plev_wap; README

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QusijEwmX4bwsbKvYikBaV
</commit_message>
<xml_diff>
--- a/CORDEX_Cmor_variables.xlsx
+++ b/CORDEX_Cmor_variables.xlsx
@@ -19985,58 +19985,58 @@
       </c>
     </row>
     <row r="317">
-      <c r="A317" s="4" t="inlineStr">
+      <c r="A317" t="inlineStr">
         <is>
           <t>wap</t>
         </is>
       </c>
-      <c r="B317" s="4" t="inlineStr">
+      <c r="B317" t="inlineStr">
         <is>
           <t>FPS-LUCAS</t>
         </is>
       </c>
-      <c r="C317" s="4" t="inlineStr">
+      <c r="C317" t="inlineStr">
         <is>
           <t>TIER 1</t>
         </is>
       </c>
-      <c r="D317" s="4" t="inlineStr">
+      <c r="D317" t="inlineStr">
         <is>
           <t>Pa s-1</t>
         </is>
       </c>
-      <c r="E317" s="5" t="inlineStr">
-        <is>
-          <t>i</t>
-        </is>
-      </c>
-      <c r="F317" s="5" t="inlineStr"/>
-      <c r="G317" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="H317" s="5" t="inlineStr"/>
-      <c r="I317" s="5" t="inlineStr"/>
-      <c r="J317" s="5" t="inlineStr"/>
-      <c r="K317" s="4" t="inlineStr">
+      <c r="E317" s="3" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
+      </c>
+      <c r="F317" s="3" t="inlineStr"/>
+      <c r="G317" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H317" s="3" t="inlineStr"/>
+      <c r="I317" s="3" t="inlineStr"/>
+      <c r="J317" s="3" t="inlineStr"/>
+      <c r="K317" t="inlineStr">
         <is>
           <t>omega</t>
         </is>
       </c>
-      <c r="L317" s="4" t="inlineStr">
+      <c r="L317" t="inlineStr">
         <is>
           <t>lagrangian_tendency_of_air_pressure</t>
         </is>
       </c>
-      <c r="M317" s="4" t="inlineStr">
-        <is>
-          <t>W P PB T QVAPOR</t>
-        </is>
-      </c>
-      <c r="N317" s="4" t="inlineStr">
-        <is>
-          <t>not produced by CORDEX_Cmor; header ready; omega = -rho g w on pressure levels</t>
+      <c r="M317" t="inlineStr">
+        <is>
+          <t>W T QVAPOR P PB</t>
+        </is>
+      </c>
+      <c r="N317" t="inlineStr">
+        <is>
+          <t>CORDEX_Cmor: RCM_plev_wap (plev_wap varset), as wap&lt;p&gt; on each pressure level (1000 to 30 hPa); omega = -rho g w; written every 6 h</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wind gust programs (UPP and Brasseur/CDXWRF); hfso, clgvi, clhvi in the varsets; compile fixes
- RCM_sfc_wsgsmax: daily maximum of the hourly gust with the UPP formula of
  the old RCM_50km_sfc_gust_era.f90 (heights above ground, grid-point
  indices, level defined below the first model level)
- RCM_sfc_wsgsmax_b01: Brasseur (2001) as gustwind_Brasseur01 of the
  CORDEX-WRF module (LluisFB/WRF, branch cdxwrf); needs TKE_PBL
- gust varset (RCM_sfc_wsgsmax; the b01 line commented), wpth4 varset
  (clgvi, clhvi), hfso in out2; TIME, ADVANCE_YEAR, NEXT
- RCM_sfc_hfso: hourly mean of GRDFLX as RCM_sfc_hfls (was instantaneous
  with 'time: mean')
- RCM_plev_wa / RCM_plev_wap: allocate w (and t, qv) of datvar_s (they
  allocated the removed wa_ws / wp_w and did not compile)
- headers, aggregation rows, variable list, README

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QusijEwmX4bwsbKvYikBaV
</commit_message>
<xml_diff>
--- a/CORDEX_Cmor_variables.xlsx
+++ b/CORDEX_Cmor_variables.xlsx
@@ -1522,11 +1522,7 @@
       <c r="F17" s="3" t="inlineStr"/>
       <c r="G17" s="3" t="inlineStr"/>
       <c r="H17" s="3" t="inlineStr"/>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>x¹</t>
-        </is>
-      </c>
+      <c r="I17" s="3" t="inlineStr"/>
       <c r="J17" s="3" t="inlineStr"/>
       <c r="K17" s="3" t="inlineStr">
         <is>
@@ -1579,11 +1575,7 @@
       <c r="F18" s="3" t="inlineStr"/>
       <c r="G18" s="3" t="inlineStr"/>
       <c r="H18" s="3" t="inlineStr"/>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>x¹</t>
-        </is>
-      </c>
+      <c r="I18" s="3" t="inlineStr"/>
       <c r="J18" s="3" t="inlineStr"/>
       <c r="K18" s="3" t="inlineStr">
         <is>
@@ -4029,132 +4021,132 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="inlineStr">
+      <c r="A56" t="inlineStr">
         <is>
           <t>clgvi</t>
         </is>
       </c>
-      <c r="B56" s="4" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>CORDEX-CMIP6</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>TIER 1</t>
         </is>
       </c>
-      <c r="D56" s="4" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t>kg m-2</t>
         </is>
       </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>i</t>
-        </is>
-      </c>
-      <c r="F56" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="G56" s="5" t="inlineStr"/>
-      <c r="H56" s="5" t="inlineStr"/>
-      <c r="I56" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="J56" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="K56" s="5" t="inlineStr"/>
-      <c r="L56" s="4" t="inlineStr">
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr"/>
+      <c r="H56" s="3" t="inlineStr"/>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr"/>
+      <c r="L56" t="inlineStr">
         <is>
           <t>Vertical integral of mass content of graupel</t>
         </is>
       </c>
-      <c r="M56" s="4" t="inlineStr">
+      <c r="M56" t="inlineStr">
         <is>
           <t>atmosphere_mass_content_of_graupel</t>
         </is>
       </c>
-      <c r="N56" s="4" t="inlineStr">
+      <c r="N56" t="inlineStr">
         <is>
           <t>QGRAUP P PB PSFC</t>
         </is>
       </c>
-      <c r="O56" s="4" t="inlineStr">
-        <is>
-          <t>not produced by CORDEX_Cmor; header ready; vertical integral</t>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>CORDEX_Cmor: RCM_sfc_clgvi (wpth4 varset)</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="4" t="inlineStr">
+      <c r="A57" t="inlineStr">
         <is>
           <t>clhvi</t>
         </is>
       </c>
-      <c r="B57" s="4" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>CORDEX-CMIP6</t>
         </is>
       </c>
-      <c r="C57" s="4" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>TIER 1</t>
         </is>
       </c>
-      <c r="D57" s="4" t="inlineStr">
+      <c r="D57" t="inlineStr">
         <is>
           <t>kg m-2</t>
         </is>
       </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>i</t>
-        </is>
-      </c>
-      <c r="F57" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="G57" s="5" t="inlineStr"/>
-      <c r="H57" s="5" t="inlineStr"/>
-      <c r="I57" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="J57" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="K57" s="5" t="inlineStr"/>
-      <c r="L57" s="4" t="inlineStr">
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr"/>
+      <c r="H57" s="3" t="inlineStr"/>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr"/>
+      <c r="L57" t="inlineStr">
         <is>
           <t>Vertical integral of mass content of hail</t>
         </is>
       </c>
-      <c r="M57" s="4" t="inlineStr">
+      <c r="M57" t="inlineStr">
         <is>
           <t>atmosphere_mass_content_of_hail</t>
         </is>
       </c>
-      <c r="N57" s="4" t="inlineStr">
+      <c r="N57" t="inlineStr">
         <is>
           <t>QHAIL P PB PSFC</t>
         </is>
       </c>
-      <c r="O57" s="4" t="inlineStr">
-        <is>
-          <t>not produced by CORDEX_Cmor; header ready; vertical integral (2-moment microphysics with hail)</t>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>CORDEX_Cmor: RCM_sfc_clhvi (wpth4 varset); needs a microphysics with hail (QHAIL)</t>
         </is>
       </c>
     </row>
@@ -8944,59 +8936,59 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="4" t="inlineStr">
+      <c r="A127" t="inlineStr">
         <is>
           <t>wsgsmax</t>
         </is>
       </c>
-      <c r="B127" s="4" t="inlineStr">
+      <c r="B127" t="inlineStr">
         <is>
           <t>CORDEX-CMIP6</t>
         </is>
       </c>
-      <c r="C127" s="4" t="inlineStr">
+      <c r="C127" t="inlineStr">
         <is>
           <t>TIER 2</t>
         </is>
       </c>
-      <c r="D127" s="4" t="inlineStr">
+      <c r="D127" t="inlineStr">
         <is>
           <t>m s-1</t>
         </is>
       </c>
-      <c r="E127" s="5" t="inlineStr"/>
-      <c r="F127" s="5" t="inlineStr"/>
-      <c r="G127" s="5" t="inlineStr"/>
-      <c r="H127" s="5" t="inlineStr"/>
-      <c r="I127" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="J127" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="K127" s="5" t="inlineStr"/>
-      <c r="L127" s="4" t="inlineStr">
+      <c r="E127" s="3" t="inlineStr"/>
+      <c r="F127" s="3" t="inlineStr"/>
+      <c r="G127" s="3" t="inlineStr"/>
+      <c r="H127" s="3" t="inlineStr"/>
+      <c r="I127" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J127" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K127" s="3" t="inlineStr"/>
+      <c r="L127" t="inlineStr">
         <is>
           <t>Daily Maximum Near-Surface Wind Speed of Gust</t>
         </is>
       </c>
-      <c r="M127" s="4" t="inlineStr">
+      <c r="M127" t="inlineStr">
         <is>
           <t>wind_speed_of_gust</t>
         </is>
       </c>
-      <c r="N127" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O127" s="4" t="inlineStr">
-        <is>
-          <t>not produced by CORDEX_Cmor; header ready; no gust diagnostic in the WRF output</t>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t>U10 V10 U V PH PHB HGT PBLH (b01: also T QVAPOR QCLOUD TKE_PBL)</t>
+        </is>
+      </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>CORDEX_Cmor: RCM_sfc_wsgsmax (gust varset), UPP formula, or RCM_sfc_wsgsmax_b01, Brasseur 2001 as CDXWRF; daily maximum of the hourly gust</t>
         </is>
       </c>
     </row>
@@ -13597,11 +13589,7 @@
       <c r="F196" s="3" t="inlineStr"/>
       <c r="G196" s="3" t="inlineStr"/>
       <c r="H196" s="3" t="inlineStr"/>
-      <c r="I196" s="3" t="inlineStr">
-        <is>
-          <t>x¹</t>
-        </is>
-      </c>
+      <c r="I196" s="3" t="inlineStr"/>
       <c r="J196" s="3" t="inlineStr"/>
       <c r="K196" s="3" t="inlineStr">
         <is>
@@ -13923,11 +13911,7 @@
       <c r="F202" s="5" t="inlineStr"/>
       <c r="G202" s="5" t="inlineStr"/>
       <c r="H202" s="5" t="inlineStr"/>
-      <c r="I202" s="5" t="inlineStr">
-        <is>
-          <t>x¹</t>
-        </is>
-      </c>
+      <c r="I202" s="5" t="inlineStr"/>
       <c r="J202" s="5" t="inlineStr"/>
       <c r="K202" s="5" t="inlineStr">
         <is>
@@ -13956,67 +13940,67 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="4" t="inlineStr">
+      <c r="A203" t="inlineStr">
         <is>
           <t>hfso</t>
         </is>
       </c>
-      <c r="B203" s="4" t="inlineStr">
+      <c r="B203" t="inlineStr">
         <is>
           <t>CORDEX-CMIP6</t>
         </is>
       </c>
-      <c r="C203" s="4" t="inlineStr">
+      <c r="C203" t="inlineStr">
         <is>
           <t>TIER 2</t>
         </is>
       </c>
-      <c r="D203" s="4" t="inlineStr">
+      <c r="D203" t="inlineStr">
         <is>
           <t>W m-2</t>
         </is>
       </c>
-      <c r="E203" s="5" t="inlineStr">
+      <c r="E203" s="3" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="F203" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="G203" s="5" t="inlineStr"/>
-      <c r="H203" s="5" t="inlineStr"/>
-      <c r="I203" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="J203" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="K203" s="5" t="inlineStr"/>
-      <c r="L203" s="4" t="inlineStr">
+      <c r="F203" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="G203" s="3" t="inlineStr"/>
+      <c r="H203" s="3" t="inlineStr"/>
+      <c r="I203" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J203" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K203" s="3" t="inlineStr"/>
+      <c r="L203" t="inlineStr">
         <is>
           <t>Surface Downward Ground Heat Flux</t>
         </is>
       </c>
-      <c r="M203" s="4" t="inlineStr">
+      <c r="M203" t="inlineStr">
         <is>
           <t>surface_downward_ground_heat_flux</t>
         </is>
       </c>
-      <c r="N203" s="4" t="inlineStr">
+      <c r="N203" t="inlineStr">
         <is>
           <t>GRDFLX</t>
         </is>
       </c>
-      <c r="O203" s="4" t="inlineStr">
-        <is>
-          <t>not produced by CORDEX_Cmor; header ready</t>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>CORDEX_Cmor: RCM_sfc_hfso (out2 varset); hourly mean of GRDFLX (positive into the soil)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wind gust: one program, Brasseur (2001) if QKE is in wrfout, else UPP
RCM_sfc_wsgsmax checks the first wrfout file of the job for QKE: with it,
the Brasseur/CDXWRF gust (reads T, QVAPOR, QCLOUD, QKE); without it, the
UPP formula. The method is written to the log. RCM_sfc_wsgsmax_b01.f90
removed (merged), gust_b01 flag in datvar_s; varsets, header, README,
variable list.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QusijEwmX4bwsbKvYikBaV
</commit_message>
<xml_diff>
--- a/CORDEX_Cmor_variables.xlsx
+++ b/CORDEX_Cmor_variables.xlsx
@@ -8983,12 +8983,12 @@
       </c>
       <c r="N127" t="inlineStr">
         <is>
-          <t>U10 V10 U V PH PHB HGT PBLH (b01: also T QVAPOR QCLOUD QKE)</t>
+          <t>U10 V10 U V PH PHB HGT PBLH T QVAPOR QCLOUD QKE</t>
         </is>
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_wsgsmax (gust varset), UPP formula, or RCM_sfc_wsgsmax_b01, Brasseur 2001 as CDXWRF; daily maximum of the hourly gust</t>
+          <t>CORDEX_Cmor: RCM_sfc_wsgsmax (gust varset); Brasseur 2001 as CDXWRF if QKE is in wrfout (T QVAPOR QCLOUD QKE), else UPP formula (U10 V10); daily maximum of the hourly gust</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
areacella and rootd (fx)
- RCM_fx_areacella: DX*DY/(MAPFAC_MX*MAPFAC_MY) of the geo_em file
  (MAPFAC_M if no MX/MY; dx_val/dy_val if no DX/DY attributes)
- RCM_fx_rootd: sum of the top NROOT soil layers (sdepth) of the dominant
  class (LU_INDEX), NROOT of WRF VEGPARM.TBL / Noah-MP NoahmpTable.TBL for
  MODIS and USGS (LCZ as urban, lakes 0); sea missing
- datvar_s: nroot_modis, nroot_usgs, msftx, msfty, dx_geo, dy_geo, fx_exists
- fx varset, headers, README, variable list

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QusijEwmX4bwsbKvYikBaV
</commit_message>
<xml_diff>
--- a/CORDEX_Cmor_variables.xlsx
+++ b/CORDEX_Cmor_variables.xlsx
@@ -13675,55 +13675,51 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="4" t="inlineStr">
+      <c r="A198" t="inlineStr">
         <is>
           <t>rootd</t>
         </is>
       </c>
-      <c r="B198" s="4" t="inlineStr">
+      <c r="B198" t="inlineStr">
         <is>
           <t>CORDEX-CMIP6</t>
         </is>
       </c>
-      <c r="C198" s="4" t="inlineStr">
+      <c r="C198" t="inlineStr">
         <is>
           <t>TIER 2</t>
         </is>
       </c>
-      <c r="D198" s="4" t="inlineStr">
+      <c r="D198" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="E198" s="5" t="inlineStr"/>
-      <c r="F198" s="5" t="inlineStr"/>
-      <c r="G198" s="5" t="inlineStr"/>
-      <c r="H198" s="5" t="inlineStr"/>
-      <c r="I198" s="5" t="inlineStr"/>
-      <c r="J198" s="5" t="inlineStr"/>
-      <c r="K198" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="L198" s="4" t="inlineStr">
+      <c r="E198" s="3" t="inlineStr"/>
+      <c r="F198" s="3" t="inlineStr"/>
+      <c r="G198" s="3" t="inlineStr"/>
+      <c r="H198" s="3" t="inlineStr"/>
+      <c r="I198" s="3" t="inlineStr"/>
+      <c r="J198" s="3" t="inlineStr"/>
+      <c r="K198" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="L198" t="inlineStr">
         <is>
           <t>Maximum Root Depth</t>
         </is>
       </c>
-      <c r="M198" s="4" t="inlineStr">
+      <c r="M198" t="inlineStr">
         <is>
           <t>root_depth</t>
         </is>
       </c>
-      <c r="N198" s="4" t="inlineStr">
-        <is>
-          <t>LU_INDEX ZS DZS</t>
-        </is>
-      </c>
-      <c r="O198" s="4" t="inlineStr">
-        <is>
-          <t>not produced by CORDEX_Cmor; header ready; root layers per vegetation class (NROOT of VEGPARM.TBL)</t>
+      <c r="N198" t="inlineStr"/>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>CORDEX_Cmor: RCM_fx_rootd (fx varset); sum of the top NROOT soil layers (VEGPARM.TBL NROOT of the dominant class, LU_INDEX of geo_em)</t>
         </is>
       </c>
     </row>
@@ -13887,55 +13883,55 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="4" t="inlineStr">
+      <c r="A202" t="inlineStr">
         <is>
           <t>areacella</t>
         </is>
       </c>
-      <c r="B202" s="4" t="inlineStr">
+      <c r="B202" t="inlineStr">
         <is>
           <t>CORDEX-CMIP6, FPS-LUCAS</t>
         </is>
       </c>
-      <c r="C202" s="4" t="inlineStr">
+      <c r="C202" t="inlineStr">
         <is>
           <t>TIER 2; LUCAS CORE</t>
         </is>
       </c>
-      <c r="D202" s="4" t="inlineStr">
+      <c r="D202" t="inlineStr">
         <is>
           <t>m2</t>
         </is>
       </c>
-      <c r="E202" s="5" t="inlineStr"/>
-      <c r="F202" s="5" t="inlineStr"/>
-      <c r="G202" s="5" t="inlineStr"/>
-      <c r="H202" s="5" t="inlineStr"/>
-      <c r="I202" s="5" t="inlineStr"/>
-      <c r="J202" s="5" t="inlineStr"/>
-      <c r="K202" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="L202" s="4" t="inlineStr">
+      <c r="E202" s="3" t="inlineStr"/>
+      <c r="F202" s="3" t="inlineStr"/>
+      <c r="G202" s="3" t="inlineStr"/>
+      <c r="H202" s="3" t="inlineStr"/>
+      <c r="I202" s="3" t="inlineStr"/>
+      <c r="J202" s="3" t="inlineStr"/>
+      <c r="K202" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr">
         <is>
           <t>Atmosphere Grid-Cell Area</t>
         </is>
       </c>
-      <c r="M202" s="4" t="inlineStr">
+      <c r="M202" t="inlineStr">
         <is>
           <t>cell_area</t>
         </is>
       </c>
-      <c r="N202" s="4" t="inlineStr">
-        <is>
-          <t>MAPFAC_MX MAPFAC_MY</t>
-        </is>
-      </c>
-      <c r="O202" s="4" t="inlineStr">
-        <is>
-          <t>not produced by CORDEX_Cmor; header ready; geo_em; DX*DY/(MAPFAC_MX*MAPFAC_MY) with the DX/DY attributes</t>
+      <c r="N202" t="inlineStr">
+        <is>
+          <t>MAPFAC_MX MAPFAC_MY MAPFAC_M</t>
+        </is>
+      </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>CORDEX_Cmor: RCM_fx_areacella (fx varset); DX*DY/(MAPFAC_MX*MAPFAC_MY) of the geo_em file</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Variable list: rootd fields
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QusijEwmX4bwsbKvYikBaV
</commit_message>
<xml_diff>
--- a/CORDEX_Cmor_variables.xlsx
+++ b/CORDEX_Cmor_variables.xlsx
@@ -13716,10 +13716,14 @@
           <t>root_depth</t>
         </is>
       </c>
-      <c r="N198" t="inlineStr"/>
+      <c r="N198" t="inlineStr">
+        <is>
+          <t>LU_INDEX LANDMASK</t>
+        </is>
+      </c>
       <c r="O198" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_fx_rootd (fx varset); sum of the top NROOT soil layers (VEGPARM.TBL NROOT of the dominant class, LU_INDEX of geo_em)</t>
+          <t>CORDEX_Cmor: RCM_fx_rootd (fx varset); from geo_em; sum of the top NROOT soil layers (VEGPARM.TBL NROOT of the dominant class, LU_INDEX of geo_em)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Split RCM_sfc_lsmflx into RCM_sfc_evspsblsoi, RCM_sfc_evspsblveg, RCM_sfc_tran
- One program per variable, as RCM_sfc_hfls: the field (EDIR, ECAN, ETRAN) is wrfvar
  of the header; hourly mean of the rates at the start and end of each hour, sea
  points missing (huge_val).
- No local declarations: the current and previous rates are wrfv2D and outvar_i of
  datvar_s (the old la_rate, la_ratep, la_ratev and read_field are gone).
- varsets (all three): lsm uses RCM_sfc_VAR:evspsblsoi,evspsblveg,tran.
- Header comments, README and the variable list updated; RCM_sfc_lsmflx.f90 removed.
- Output identical to RCM_sfc_lsmflx (data, attributes, file names; test month).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QusijEwmX4bwsbKvYikBaV
</commit_message>
<xml_diff>
--- a/CORDEX_Cmor_variables.xlsx
+++ b/CORDEX_Cmor_variables.xlsx
@@ -15419,7 +15419,7 @@
       </c>
       <c r="O226" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_lsmflx (lsm varset)</t>
+          <t>CORDEX_Cmor: RCM_sfc_evspsblsoi (lsm varset)</t>
         </is>
       </c>
     </row>
@@ -15476,7 +15476,7 @@
       </c>
       <c r="O227" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_lsmflx (lsm varset)</t>
+          <t>CORDEX_Cmor: RCM_sfc_evspsblveg (lsm varset)</t>
         </is>
       </c>
     </row>
@@ -16787,7 +16787,7 @@
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_lsmflx (lsm varset)</t>
+          <t>CORDEX_Cmor: RCM_sfc_tran (lsm varset)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Split RCM_sfc_lsm into RCM_sfc_lai, RCM_sfc_vegFrac, RCM_sfc_alb
- One program per variable reading wrfvar of the header (LAI, FVEG, ALBEDO);
  same masking (lai, vegFrac: sea missing), scaling (vegFrac to %) and rounding
  to 1e-4 as before.
- No local declarations left (ls_v, ls_scale, ls_land gone); missing value is
  huge_val of datvar_s.
- varsets (all three): lsm = RCM_sfc_VAR:evspsblsoi,evspsblveg,tran,lai,vegFrac,alb.
- README and the variable list updated; RCM_sfc_lsm.f90 removed.
- Output identical to RCM_sfc_lsm (data, attributes, file names; test month).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QusijEwmX4bwsbKvYikBaV
</commit_message>
<xml_diff>
--- a/CORDEX_Cmor_variables.xlsx
+++ b/CORDEX_Cmor_variables.xlsx
@@ -15020,7 +15020,7 @@
       </c>
       <c r="O219" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_lsm (lsm varset); LUCAS name LAI</t>
+          <t>CORDEX_Cmor: RCM_sfc_lai (lsm varset); LUCAS name LAI</t>
         </is>
       </c>
     </row>
@@ -15077,7 +15077,7 @@
       </c>
       <c r="O220" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_lsm (lsm varset)</t>
+          <t>CORDEX_Cmor: RCM_sfc_alb (lsm varset)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Relative vorticity on pressure levels; hu left out
- RCM_plev_vortmen (varsets plev_vortmen0, plev_vortmen1, not in ORDER):
  vortmen<p> on the pressure levels of the other plev variables, every wp_step
  hours; zeta = m^2 [d(v/m_v)/dx - d(u/m_u)/dy] on the model levels as wrf-python
  (centred differences, one-cell halo around the window), interpolated in log(p)
  as RCM_plev_wap. Headers vortmen1000 ... vortmen10 (generic header_vortmen removed).
- datvar_s: vo_mu, vo_mv, vo_mt, vo_dx, vo_dy, vo_dudy, vo_dvdx, halo sizes and indices.
- hu removed from the variable list (and header_hu).
- snw: the CORDEX-CMIP6 tables ask for 6hr (point), day and mon only, so its
  header and program are left unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QusijEwmX4bwsbKvYikBaV
</commit_message>
<xml_diff>
--- a/CORDEX_Cmor_variables.xlsx
+++ b/CORDEX_Cmor_variables.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="variables" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'variables'!$A$1:$O$260</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'variables'!$A$1:$O$259</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O262"/>
+  <dimension ref="A1:O261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -14911,66 +14911,66 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="4" t="inlineStr">
-        <is>
-          <t>hu</t>
-        </is>
-      </c>
-      <c r="B218" s="4" t="inlineStr">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>lai</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
         <is>
           <t>FPS-LUCAS</t>
         </is>
       </c>
-      <c r="C218" s="4" t="inlineStr">
+      <c r="C218" t="inlineStr">
         <is>
           <t>CORE</t>
         </is>
       </c>
-      <c r="D218" s="4" t="inlineStr">
-        <is>
-          <t>m3/m3</t>
-        </is>
-      </c>
-      <c r="E218" s="5" t="inlineStr">
-        <is>
-          <t>i</t>
-        </is>
-      </c>
-      <c r="F218" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="G218" s="5" t="inlineStr"/>
-      <c r="H218" s="5" t="inlineStr"/>
-      <c r="I218" s="5" t="inlineStr"/>
-      <c r="J218" s="5" t="inlineStr"/>
-      <c r="K218" s="5" t="inlineStr"/>
-      <c r="L218" s="4" t="inlineStr">
-        <is>
-          <t>Atmospheric humidity at model levels</t>
-        </is>
-      </c>
-      <c r="M218" s="4" t="inlineStr">
-        <is>
-          <t>specific_humidity</t>
-        </is>
-      </c>
-      <c r="N218" s="4" t="inlineStr">
-        <is>
-          <t>QVAPOR</t>
-        </is>
-      </c>
-      <c r="O218" s="4" t="inlineStr">
-        <is>
-          <t>not produced by CORDEX_Cmor; header ready; model levels</t>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E218" s="3" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
+      </c>
+      <c r="F218" s="3" t="inlineStr"/>
+      <c r="G218" s="3" t="inlineStr"/>
+      <c r="H218" s="3" t="inlineStr"/>
+      <c r="I218" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J218" s="3" t="inlineStr"/>
+      <c r="K218" s="3" t="inlineStr"/>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t>leaf area index</t>
+        </is>
+      </c>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>leaf_area_index</t>
+        </is>
+      </c>
+      <c r="N218" t="inlineStr">
+        <is>
+          <t>LAI</t>
+        </is>
+      </c>
+      <c r="O218" t="inlineStr">
+        <is>
+          <t>CORDEX_Cmor: RCM_sfc_lai (lsm varset); LUCAS name LAI</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>lai</t>
+          <t>alb</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -14980,7 +14980,7 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>TIER 1</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
@@ -15005,143 +15005,143 @@
       <c r="K219" s="3" t="inlineStr"/>
       <c r="L219" t="inlineStr">
         <is>
-          <t>leaf area index</t>
+          <t>Albedo</t>
         </is>
       </c>
       <c r="M219" t="inlineStr">
         <is>
-          <t>leaf_area_index</t>
+          <t>surface_albedo</t>
         </is>
       </c>
       <c r="N219" t="inlineStr">
         <is>
-          <t>LAI</t>
+          <t>ALBEDO</t>
         </is>
       </c>
       <c r="O219" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_lai (lsm varset); LUCAS name LAI</t>
+          <t>CORDEX_Cmor: RCM_sfc_alb (lsm varset)</t>
         </is>
       </c>
     </row>
     <row r="220">
-      <c r="A220" t="inlineStr">
-        <is>
-          <t>alb</t>
-        </is>
-      </c>
-      <c r="B220" t="inlineStr">
+      <c r="A220" s="4" t="inlineStr">
+        <is>
+          <t>albc</t>
+        </is>
+      </c>
+      <c r="B220" s="4" t="inlineStr">
         <is>
           <t>FPS-LUCAS</t>
         </is>
       </c>
-      <c r="C220" t="inlineStr">
+      <c r="C220" s="4" t="inlineStr">
         <is>
           <t>TIER 1</t>
         </is>
       </c>
-      <c r="D220" t="inlineStr">
+      <c r="D220" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E220" s="3" t="inlineStr">
-        <is>
-          <t>i</t>
-        </is>
-      </c>
-      <c r="F220" s="3" t="inlineStr"/>
-      <c r="G220" s="3" t="inlineStr"/>
-      <c r="H220" s="3" t="inlineStr"/>
-      <c r="I220" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="J220" s="3" t="inlineStr"/>
-      <c r="K220" s="3" t="inlineStr"/>
-      <c r="L220" t="inlineStr">
-        <is>
-          <t>Albedo</t>
-        </is>
-      </c>
-      <c r="M220" t="inlineStr">
-        <is>
-          <t>surface_albedo</t>
-        </is>
-      </c>
-      <c r="N220" t="inlineStr">
-        <is>
-          <t>ALBEDO</t>
-        </is>
-      </c>
-      <c r="O220" t="inlineStr">
-        <is>
-          <t>CORDEX_Cmor: RCM_sfc_alb (lsm varset)</t>
+      <c r="E220" s="5" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
+      </c>
+      <c r="F220" s="5" t="inlineStr"/>
+      <c r="G220" s="5" t="inlineStr"/>
+      <c r="H220" s="5" t="inlineStr"/>
+      <c r="I220" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J220" s="5" t="inlineStr"/>
+      <c r="K220" s="5" t="inlineStr"/>
+      <c r="L220" s="4" t="inlineStr">
+        <is>
+          <t>Albedo of the vegetation: fraction of incoming solar radiation which is reflected before reaching the ground.</t>
+        </is>
+      </c>
+      <c r="M220" s="4" t="inlineStr">
+        <is>
+          <t>canopy_albedo</t>
+        </is>
+      </c>
+      <c r="N220" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O220" s="4" t="inlineStr">
+        <is>
+          <t>not produced by CORDEX_Cmor; header ready; no canopy albedo in the WRF output</t>
         </is>
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="4" t="inlineStr">
-        <is>
-          <t>albc</t>
-        </is>
-      </c>
-      <c r="B221" s="4" t="inlineStr">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>baresoilFrac</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
         <is>
           <t>FPS-LUCAS</t>
         </is>
       </c>
-      <c r="C221" s="4" t="inlineStr">
+      <c r="C221" t="inlineStr">
         <is>
           <t>TIER 1</t>
         </is>
       </c>
-      <c r="D221" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E221" s="5" t="inlineStr">
-        <is>
-          <t>i</t>
-        </is>
-      </c>
-      <c r="F221" s="5" t="inlineStr"/>
-      <c r="G221" s="5" t="inlineStr"/>
-      <c r="H221" s="5" t="inlineStr"/>
-      <c r="I221" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="J221" s="5" t="inlineStr"/>
-      <c r="K221" s="5" t="inlineStr"/>
-      <c r="L221" s="4" t="inlineStr">
-        <is>
-          <t>Albedo of the vegetation: fraction of incoming solar radiation which is reflected before reaching the ground.</t>
-        </is>
-      </c>
-      <c r="M221" s="4" t="inlineStr">
-        <is>
-          <t>canopy_albedo</t>
-        </is>
-      </c>
-      <c r="N221" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O221" s="4" t="inlineStr">
-        <is>
-          <t>not produced by CORDEX_Cmor; header ready; no canopy albedo in the WRF output</t>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E221" s="3" t="inlineStr"/>
+      <c r="F221" s="3" t="inlineStr"/>
+      <c r="G221" s="3" t="inlineStr"/>
+      <c r="H221" s="3" t="inlineStr"/>
+      <c r="I221" s="3" t="inlineStr">
+        <is>
+          <t>x¹</t>
+        </is>
+      </c>
+      <c r="J221" s="3" t="inlineStr"/>
+      <c r="K221" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="L221" t="inlineStr">
+        <is>
+          <t>Bare Soil Percentage Area Coverage</t>
+        </is>
+      </c>
+      <c r="M221" t="inlineStr">
+        <is>
+          <t>area_fraction</t>
+        </is>
+      </c>
+      <c r="N221" t="inlineStr">
+        <is>
+          <t>LANDUSEF</t>
+        </is>
+      </c>
+      <c r="O221" t="inlineStr">
+        <is>
+          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF classes grouped (landuse_field in shared_subs_v2.f90)</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>baresoilFrac</t>
+          <t>cnc</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -15176,7 +15176,7 @@
       </c>
       <c r="L222" t="inlineStr">
         <is>
-          <t>Bare Soil Percentage Area Coverage</t>
+          <t>Percentage of area covered by vegetation.</t>
         </is>
       </c>
       <c r="M222" t="inlineStr">
@@ -15191,14 +15191,14 @@
       </c>
       <c r="O222" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF classes grouped (landuse_field in shared_subs_v2.f90)</t>
+          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF tree+shrub+grass+crop (landuse_field in shared_subs_v2.f90)</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>cnc</t>
+          <t>cropFrac</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -15233,7 +15233,7 @@
       </c>
       <c r="L223" t="inlineStr">
         <is>
-          <t>Percentage of area covered by vegetation.</t>
+          <t>Percentage Crop Cover</t>
         </is>
       </c>
       <c r="M223" t="inlineStr">
@@ -15248,14 +15248,14 @@
       </c>
       <c r="O223" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF tree+shrub+grass+crop (landuse_field in shared_subs_v2.f90)</t>
+          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF classes grouped (landuse_field in shared_subs_v2.f90)</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>cropFrac</t>
+          <t>cVeg</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -15270,49 +15270,49 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E224" s="3" t="inlineStr"/>
+          <t>kg m-2</t>
+        </is>
+      </c>
+      <c r="E224" s="3" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
+      </c>
       <c r="F224" s="3" t="inlineStr"/>
       <c r="G224" s="3" t="inlineStr"/>
       <c r="H224" s="3" t="inlineStr"/>
       <c r="I224" s="3" t="inlineStr">
         <is>
-          <t>x¹</t>
+          <t>x</t>
         </is>
       </c>
       <c r="J224" s="3" t="inlineStr"/>
-      <c r="K224" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K224" s="3" t="inlineStr"/>
       <c r="L224" t="inlineStr">
         <is>
-          <t>Percentage Crop Cover</t>
+          <t>Carbon mass per unit area in vegetation.</t>
         </is>
       </c>
       <c r="M224" t="inlineStr">
         <is>
-          <t>area_fraction</t>
+          <t>vegetation_carbon_content</t>
         </is>
       </c>
       <c r="N224" t="inlineStr">
         <is>
-          <t>LANDUSEF</t>
+          <t>LFMASS RTMASS STMASS WOOD</t>
         </is>
       </c>
       <c r="O224" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF classes grouped (landuse_field in shared_subs_v2.f90)</t>
+          <t>CORDEX_Cmor: RCM_sfc_cVeg (lsm varset); meaningful with Noah-MP dynamic vegetation (opt_dveg) only</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>cVeg</t>
+          <t>evspsblsoi</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -15327,49 +15327,49 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>kg m-2</t>
+          <t>kg m-2 s-1</t>
         </is>
       </c>
       <c r="E225" s="3" t="inlineStr">
         <is>
-          <t>i</t>
-        </is>
-      </c>
-      <c r="F225" s="3" t="inlineStr"/>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="F225" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G225" s="3" t="inlineStr"/>
       <c r="H225" s="3" t="inlineStr"/>
-      <c r="I225" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I225" s="3" t="inlineStr"/>
       <c r="J225" s="3" t="inlineStr"/>
       <c r="K225" s="3" t="inlineStr"/>
       <c r="L225" t="inlineStr">
         <is>
-          <t>Carbon mass per unit area in vegetation.</t>
+          <t>Water evaporation from soil (including sublimation).</t>
         </is>
       </c>
       <c r="M225" t="inlineStr">
         <is>
-          <t>vegetation_carbon_content</t>
+          <t>water_evaporation_flux_from_soil</t>
         </is>
       </c>
       <c r="N225" t="inlineStr">
         <is>
-          <t>LFMASS RTMASS STMASS WOOD</t>
+          <t>EDIR</t>
         </is>
       </c>
       <c r="O225" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_cVeg (lsm varset); meaningful with Noah-MP dynamic vegetation (opt_dveg) only</t>
+          <t>CORDEX_Cmor: RCM_sfc_evspsblsoi (lsm varset)</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>evspsblsoi</t>
+          <t>evspsblveg</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -15404,29 +15404,29 @@
       <c r="K226" s="3" t="inlineStr"/>
       <c r="L226" t="inlineStr">
         <is>
-          <t>Water evaporation from soil (including sublimation).</t>
+          <t>The canopy evaporation and sublimation (if present in model); may include dew formation as a negative flux.</t>
         </is>
       </c>
       <c r="M226" t="inlineStr">
         <is>
-          <t>water_evaporation_flux_from_soil</t>
+          <t>water_evaporation_flux_from_canopy</t>
         </is>
       </c>
       <c r="N226" t="inlineStr">
         <is>
-          <t>EDIR</t>
+          <t>ECAN</t>
         </is>
       </c>
       <c r="O226" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_evspsblsoi (lsm varset)</t>
+          <t>CORDEX_Cmor: RCM_sfc_evspsblveg (lsm varset)</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>evspsblveg</t>
+          <t>grassFrac</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -15441,49 +15441,49 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>kg m-2 s-1</t>
-        </is>
-      </c>
-      <c r="E227" s="3" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="F227" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E227" s="3" t="inlineStr"/>
+      <c r="F227" s="3" t="inlineStr"/>
       <c r="G227" s="3" t="inlineStr"/>
       <c r="H227" s="3" t="inlineStr"/>
-      <c r="I227" s="3" t="inlineStr"/>
+      <c r="I227" s="3" t="inlineStr">
+        <is>
+          <t>x¹</t>
+        </is>
+      </c>
       <c r="J227" s="3" t="inlineStr"/>
-      <c r="K227" s="3" t="inlineStr"/>
+      <c r="K227" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L227" t="inlineStr">
         <is>
-          <t>The canopy evaporation and sublimation (if present in model); may include dew formation as a negative flux.</t>
+          <t>Natural Grass Area Percentage</t>
         </is>
       </c>
       <c r="M227" t="inlineStr">
         <is>
-          <t>water_evaporation_flux_from_canopy</t>
+          <t>area_fraction</t>
         </is>
       </c>
       <c r="N227" t="inlineStr">
         <is>
-          <t>ECAN</t>
+          <t>LANDUSEF</t>
         </is>
       </c>
       <c r="O227" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_evspsblveg (lsm varset)</t>
+          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF classes grouped (landuse_field in shared_subs_v2.f90)</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>grassFrac</t>
+          <t>hflsLut</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -15498,49 +15498,49 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E228" s="3" t="inlineStr"/>
-      <c r="F228" s="3" t="inlineStr"/>
+          <t>W m-2</t>
+        </is>
+      </c>
+      <c r="E228" s="3" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="F228" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G228" s="3" t="inlineStr"/>
       <c r="H228" s="3" t="inlineStr"/>
-      <c r="I228" s="3" t="inlineStr">
-        <is>
-          <t>x¹</t>
-        </is>
-      </c>
+      <c r="I228" s="3" t="inlineStr"/>
       <c r="J228" s="3" t="inlineStr"/>
-      <c r="K228" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K228" s="3" t="inlineStr"/>
       <c r="L228" t="inlineStr">
         <is>
-          <t>Natural Grass Area Percentage</t>
+          <t>Latent Heat Flux on Land-Use Tile</t>
         </is>
       </c>
       <c r="M228" t="inlineStr">
         <is>
-          <t>area_fraction</t>
+          <t>surface_upward_latent_heat_flux</t>
         </is>
       </c>
       <c r="N228" t="inlineStr">
         <is>
-          <t>LANDUSEF</t>
+          <t>LH</t>
         </is>
       </c>
       <c r="O228" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF classes grouped (landuse_field in shared_subs_v2.f90)</t>
+          <t>CORDEX_Cmor: RCM_sfc_hfls (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>hflsLut</t>
+          <t>hfssLut</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -15575,29 +15575,29 @@
       <c r="K229" s="3" t="inlineStr"/>
       <c r="L229" t="inlineStr">
         <is>
-          <t>Latent Heat Flux on Land-Use Tile</t>
+          <t>Sensible Heat Flux on Land-Use Tile</t>
         </is>
       </c>
       <c r="M229" t="inlineStr">
         <is>
-          <t>surface_upward_latent_heat_flux</t>
+          <t>surface_upward_sensible_heat_flux</t>
         </is>
       </c>
       <c r="N229" t="inlineStr">
         <is>
-          <t>LH</t>
+          <t>HFX</t>
         </is>
       </c>
       <c r="O229" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_hfls (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
+          <t>CORDEX_Cmor: RCM_sfc_hfss (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>hfssLut</t>
+          <t>hussLut</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -15612,12 +15612,12 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>W m-2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E230" s="3" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>i</t>
         </is>
       </c>
       <c r="F230" s="3" t="inlineStr">
@@ -15632,29 +15632,29 @@
       <c r="K230" s="3" t="inlineStr"/>
       <c r="L230" t="inlineStr">
         <is>
-          <t>Sensible Heat Flux on Land-Use Tile</t>
+          <t>Normally, the specific humidity should be reported at the 2 meter height</t>
         </is>
       </c>
       <c r="M230" t="inlineStr">
         <is>
-          <t>surface_upward_sensible_heat_flux</t>
+          <t>specific_humidity</t>
         </is>
       </c>
       <c r="N230" t="inlineStr">
         <is>
-          <t>HFX</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="O230" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_hfss (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
+          <t>CORDEX_Cmor: RCM_sfc_huss (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>hussLut</t>
+          <t>interception</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -15669,7 +15669,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>kg m-2</t>
         </is>
       </c>
       <c r="E231" s="3" t="inlineStr">
@@ -15689,29 +15689,29 @@
       <c r="K231" s="3" t="inlineStr"/>
       <c r="L231" t="inlineStr">
         <is>
-          <t>Normally, the specific humidity should be reported at the 2 meter height</t>
+          <t>water intercepted</t>
         </is>
       </c>
       <c r="M231" t="inlineStr">
         <is>
-          <t>specific_humidity</t>
+          <t>canopy_water_amount</t>
         </is>
       </c>
       <c r="N231" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>CANLIQ CANICE</t>
         </is>
       </c>
       <c r="O231" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_huss (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
+          <t>CORDEX_Cmor: RCM_sfc_interception (lsm varset)</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>interception</t>
+          <t>irrLut</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -15726,12 +15726,12 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>kg m-2</t>
+          <t>kg m-2 s-1</t>
         </is>
       </c>
       <c r="E232" s="3" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>a</t>
         </is>
       </c>
       <c r="F232" s="3" t="inlineStr">
@@ -15746,29 +15746,29 @@
       <c r="K232" s="3" t="inlineStr"/>
       <c r="L232" t="inlineStr">
         <is>
-          <t>water intercepted</t>
+          <t>surface_downward_mass_flux_of_water_due_to_irrigation</t>
         </is>
       </c>
       <c r="M232" t="inlineStr">
         <is>
-          <t>canopy_water_amount</t>
+          <t>surface_downward_mass_flux_of_water_due_to_irrigation</t>
         </is>
       </c>
       <c r="N232" t="inlineStr">
         <is>
-          <t>CANLIQ CANICE</t>
+          <t>IRSIVOL IRMIVOL IRFIVOL</t>
         </is>
       </c>
       <c r="O232" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_interception (lsm varset)</t>
+          <t>CORDEX_Cmor: RCM_sfc_irrLut (irr varset); Noah-MP irrigation (opt_irr); add IRSIVOL IRMIVOL IRFIVOL to wrfout (iofields); no land-use tiles: grid-cell value</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>irrLut</t>
+          <t>laiLut</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -15783,49 +15783,49 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>kg m-2 s-1</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E233" s="3" t="inlineStr">
         <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="F233" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>i</t>
+        </is>
+      </c>
+      <c r="F233" s="3" t="inlineStr"/>
       <c r="G233" s="3" t="inlineStr"/>
       <c r="H233" s="3" t="inlineStr"/>
-      <c r="I233" s="3" t="inlineStr"/>
+      <c r="I233" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="J233" s="3" t="inlineStr"/>
       <c r="K233" s="3" t="inlineStr"/>
       <c r="L233" t="inlineStr">
         <is>
-          <t>surface_downward_mass_flux_of_water_due_to_irrigation</t>
+          <t>Leaf Area Index on Land-Use Tile</t>
         </is>
       </c>
       <c r="M233" t="inlineStr">
         <is>
-          <t>surface_downward_mass_flux_of_water_due_to_irrigation</t>
+          <t>leaf_area_index</t>
         </is>
       </c>
       <c r="N233" t="inlineStr">
         <is>
-          <t>IRSIVOL IRMIVOL IRFIVOL</t>
+          <t>LAI</t>
         </is>
       </c>
       <c r="O233" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_irrLut (irr varset); Noah-MP irrigation (opt_irr); add IRSIVOL IRMIVOL IRFIVOL to wrfout (iofields); no land-use tiles: grid-cell value</t>
+          <t>CORDEX_Cmor: RCM_sfc_lai (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>laiLut</t>
+          <t>landCoverFrac</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -15840,49 +15840,49 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E234" s="3" t="inlineStr">
-        <is>
-          <t>i</t>
-        </is>
-      </c>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E234" s="3" t="inlineStr"/>
       <c r="F234" s="3" t="inlineStr"/>
       <c r="G234" s="3" t="inlineStr"/>
       <c r="H234" s="3" t="inlineStr"/>
       <c r="I234" s="3" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>x¹</t>
         </is>
       </c>
       <c r="J234" s="3" t="inlineStr"/>
-      <c r="K234" s="3" t="inlineStr"/>
+      <c r="K234" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L234" t="inlineStr">
         <is>
-          <t>Leaf Area Index on Land-Use Tile</t>
+          <t>Percentage of Area by Vegetation or Land-Cover Category</t>
         </is>
       </c>
       <c r="M234" t="inlineStr">
         <is>
-          <t>leaf_area_index</t>
+          <t>area_fraction</t>
         </is>
       </c>
       <c r="N234" t="inlineStr">
         <is>
-          <t>LAI</t>
+          <t>LANDUSEF</t>
         </is>
       </c>
       <c r="O234" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_lai (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
+          <t>CORDEX_Cmor: RCM_fx_landCoverFrac (fx varset)</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>landCoverFrac</t>
+          <t>mrroLut</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -15897,49 +15897,49 @@
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E235" s="3" t="inlineStr"/>
-      <c r="F235" s="3" t="inlineStr"/>
+          <t>kg m-2 s-1</t>
+        </is>
+      </c>
+      <c r="E235" s="3" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="F235" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G235" s="3" t="inlineStr"/>
       <c r="H235" s="3" t="inlineStr"/>
-      <c r="I235" s="3" t="inlineStr">
-        <is>
-          <t>x¹</t>
-        </is>
-      </c>
+      <c r="I235" s="3" t="inlineStr"/>
       <c r="J235" s="3" t="inlineStr"/>
-      <c r="K235" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K235" s="3" t="inlineStr"/>
       <c r="L235" t="inlineStr">
         <is>
-          <t>Percentage of Area by Vegetation or Land-Cover Category</t>
+          <t>Total Runoff on Land-Use Tile</t>
         </is>
       </c>
       <c r="M235" t="inlineStr">
         <is>
-          <t>area_fraction</t>
+          <t>runoff_flux</t>
         </is>
       </c>
       <c r="N235" t="inlineStr">
         <is>
-          <t>LANDUSEF</t>
+          <t>RUNSB RUNSF</t>
         </is>
       </c>
       <c r="O235" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_fx_landCoverFrac (fx varset)</t>
+          <t>CORDEX_Cmor: RCM_sfc_mrro (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>mrroLut</t>
+          <t>mrsoLut</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -15954,12 +15954,12 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>kg m-2 s-1</t>
+          <t>kg m-2</t>
         </is>
       </c>
       <c r="E236" s="3" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>i</t>
         </is>
       </c>
       <c r="F236" s="3" t="inlineStr">
@@ -15974,29 +15974,29 @@
       <c r="K236" s="3" t="inlineStr"/>
       <c r="L236" t="inlineStr">
         <is>
-          <t>Total Runoff on Land-Use Tile</t>
+          <t>Total Soil Moisture on Land-Use Tile</t>
         </is>
       </c>
       <c r="M236" t="inlineStr">
         <is>
-          <t>runoff_flux</t>
+          <t>mass_content_of_water_in_soil</t>
         </is>
       </c>
       <c r="N236" t="inlineStr">
         <is>
-          <t>RUNSB RUNSF</t>
+          <t>SMOIS</t>
         </is>
       </c>
       <c r="O236" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_mrro (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
+          <t>CORDEX_Cmor: RCM_sfc_mrso (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>mrsoLut</t>
+          <t>mrsosLut</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -16031,12 +16031,12 @@
       <c r="K237" s="3" t="inlineStr"/>
       <c r="L237" t="inlineStr">
         <is>
-          <t>Total Soil Moisture on Land-Use Tile</t>
+          <t>the mass of water in all phases in a thin surface layer; integrate over uppermost 10cm</t>
         </is>
       </c>
       <c r="M237" t="inlineStr">
         <is>
-          <t>mass_content_of_water_in_soil</t>
+          <t>mass_content_of_water_in_soil_layer</t>
         </is>
       </c>
       <c r="N237" t="inlineStr">
@@ -16046,14 +16046,14 @@
       </c>
       <c r="O237" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_mrso (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
+          <t>CORDEX_Cmor: RCM_sfc_mrsos (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>mrsosLut</t>
+          <t>npp</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -16068,163 +16068,163 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>kg m-2</t>
+          <t>kg m-2 s-1</t>
         </is>
       </c>
       <c r="E238" s="3" t="inlineStr">
         <is>
-          <t>i</t>
-        </is>
-      </c>
-      <c r="F238" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="F238" s="3" t="inlineStr"/>
       <c r="G238" s="3" t="inlineStr"/>
       <c r="H238" s="3" t="inlineStr"/>
-      <c r="I238" s="3" t="inlineStr"/>
+      <c r="I238" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="J238" s="3" t="inlineStr"/>
       <c r="K238" s="3" t="inlineStr"/>
       <c r="L238" t="inlineStr">
         <is>
-          <t>the mass of water in all phases in a thin surface layer; integrate over uppermost 10cm</t>
+          <t>Net Primary Production on Land as Carbon Mass Flux</t>
         </is>
       </c>
       <c r="M238" t="inlineStr">
         <is>
-          <t>mass_content_of_water_in_soil_layer</t>
+          <t>net_primary_productivity_of_biomass_expressed_as_carbon</t>
         </is>
       </c>
       <c r="N238" t="inlineStr">
         <is>
-          <t>SMOIS</t>
+          <t>NPP</t>
         </is>
       </c>
       <c r="O238" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_mrsos (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
+          <t>CORDEX_Cmor: RCM_sfc_npp (lsm varset); meaningful with Noah-MP dynamic vegetation (opt_dveg) only</t>
         </is>
       </c>
     </row>
     <row r="239">
-      <c r="A239" t="inlineStr">
-        <is>
-          <t>npp</t>
-        </is>
-      </c>
-      <c r="B239" t="inlineStr">
+      <c r="A239" s="4" t="inlineStr">
+        <is>
+          <t>pastureFrac</t>
+        </is>
+      </c>
+      <c r="B239" s="4" t="inlineStr">
         <is>
           <t>FPS-LUCAS</t>
         </is>
       </c>
-      <c r="C239" t="inlineStr">
+      <c r="C239" s="4" t="inlineStr">
         <is>
           <t>TIER 1</t>
         </is>
       </c>
-      <c r="D239" t="inlineStr">
-        <is>
-          <t>kg m-2 s-1</t>
-        </is>
-      </c>
-      <c r="E239" s="3" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="F239" s="3" t="inlineStr"/>
-      <c r="G239" s="3" t="inlineStr"/>
-      <c r="H239" s="3" t="inlineStr"/>
-      <c r="I239" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="J239" s="3" t="inlineStr"/>
-      <c r="K239" s="3" t="inlineStr"/>
-      <c r="L239" t="inlineStr">
-        <is>
-          <t>Net Primary Production on Land as Carbon Mass Flux</t>
-        </is>
-      </c>
-      <c r="M239" t="inlineStr">
-        <is>
-          <t>net_primary_productivity_of_biomass_expressed_as_carbon</t>
-        </is>
-      </c>
-      <c r="N239" t="inlineStr">
-        <is>
-          <t>NPP</t>
-        </is>
-      </c>
-      <c r="O239" t="inlineStr">
-        <is>
-          <t>CORDEX_Cmor: RCM_sfc_npp (lsm varset); meaningful with Noah-MP dynamic vegetation (opt_dveg) only</t>
+      <c r="D239" s="4" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E239" s="5" t="inlineStr"/>
+      <c r="F239" s="5" t="inlineStr"/>
+      <c r="G239" s="5" t="inlineStr"/>
+      <c r="H239" s="5" t="inlineStr"/>
+      <c r="I239" s="5" t="inlineStr">
+        <is>
+          <t>x¹</t>
+        </is>
+      </c>
+      <c r="J239" s="5" t="inlineStr"/>
+      <c r="K239" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="L239" s="4" t="inlineStr">
+        <is>
+          <t>Percentage of Land Which Is Anthropogenic Pasture</t>
+        </is>
+      </c>
+      <c r="M239" s="4" t="inlineStr">
+        <is>
+          <t>area_fraction</t>
+        </is>
+      </c>
+      <c r="N239" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O239" s="4" t="inlineStr">
+        <is>
+          <t>not produced by CORDEX_Cmor; header ready; no pasture class in the WRF land-use tables</t>
         </is>
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="4" t="inlineStr">
-        <is>
-          <t>pastureFrac</t>
-        </is>
-      </c>
-      <c r="B240" s="4" t="inlineStr">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>residualFrac</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
         <is>
           <t>FPS-LUCAS</t>
         </is>
       </c>
-      <c r="C240" s="4" t="inlineStr">
+      <c r="C240" t="inlineStr">
         <is>
           <t>TIER 1</t>
         </is>
       </c>
-      <c r="D240" s="4" t="inlineStr">
+      <c r="D240" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E240" s="5" t="inlineStr"/>
-      <c r="F240" s="5" t="inlineStr"/>
-      <c r="G240" s="5" t="inlineStr"/>
-      <c r="H240" s="5" t="inlineStr"/>
-      <c r="I240" s="5" t="inlineStr">
+      <c r="E240" s="3" t="inlineStr"/>
+      <c r="F240" s="3" t="inlineStr"/>
+      <c r="G240" s="3" t="inlineStr"/>
+      <c r="H240" s="3" t="inlineStr"/>
+      <c r="I240" s="3" t="inlineStr">
         <is>
           <t>x¹</t>
         </is>
       </c>
-      <c r="J240" s="5" t="inlineStr"/>
-      <c r="K240" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="L240" s="4" t="inlineStr">
-        <is>
-          <t>Percentage of Land Which Is Anthropogenic Pasture</t>
-        </is>
-      </c>
-      <c r="M240" s="4" t="inlineStr">
+      <c r="J240" s="3" t="inlineStr"/>
+      <c r="K240" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="L240" t="inlineStr">
+        <is>
+          <t>Percentage of Grid Cell That Is Land but neither Vegetation Covered nor Bare Soil</t>
+        </is>
+      </c>
+      <c r="M240" t="inlineStr">
         <is>
           <t>area_fraction</t>
         </is>
       </c>
-      <c r="N240" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O240" s="4" t="inlineStr">
-        <is>
-          <t>not produced by CORDEX_Cmor; header ready; no pasture class in the WRF land-use tables</t>
+      <c r="N240" t="inlineStr">
+        <is>
+          <t>LANDUSEF</t>
+        </is>
+      </c>
+      <c r="O240" t="inlineStr">
+        <is>
+          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LUCAS name resdiualFrac</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>residualFrac</t>
+          <t>rlusLut</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -16239,49 +16239,49 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E241" s="3" t="inlineStr"/>
-      <c r="F241" s="3" t="inlineStr"/>
+          <t>W m-2</t>
+        </is>
+      </c>
+      <c r="E241" s="3" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="F241" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G241" s="3" t="inlineStr"/>
       <c r="H241" s="3" t="inlineStr"/>
-      <c r="I241" s="3" t="inlineStr">
-        <is>
-          <t>x¹</t>
-        </is>
-      </c>
+      <c r="I241" s="3" t="inlineStr"/>
       <c r="J241" s="3" t="inlineStr"/>
-      <c r="K241" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K241" s="3" t="inlineStr"/>
       <c r="L241" t="inlineStr">
         <is>
-          <t>Percentage of Grid Cell That Is Land but neither Vegetation Covered nor Bare Soil</t>
+          <t>Surface Upwelling Longwave on Land-Use Tile</t>
         </is>
       </c>
       <c r="M241" t="inlineStr">
         <is>
-          <t>area_fraction</t>
+          <t>surface_upwelling_longwave_flux_in_air</t>
         </is>
       </c>
       <c r="N241" t="inlineStr">
         <is>
-          <t>LANDUSEF</t>
+          <t>ACLWUPB I_ACLWUPB</t>
         </is>
       </c>
       <c r="O241" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LUCAS name resdiualFrac</t>
+          <t>CORDEX_Cmor: RCM_sfc_rad (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>rlusLut</t>
+          <t>rough</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -16296,49 +16296,49 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>W m-2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E242" s="3" t="inlineStr">
         <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="F242" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>i</t>
+        </is>
+      </c>
+      <c r="F242" s="3" t="inlineStr"/>
       <c r="G242" s="3" t="inlineStr"/>
       <c r="H242" s="3" t="inlineStr"/>
-      <c r="I242" s="3" t="inlineStr"/>
+      <c r="I242" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="J242" s="3" t="inlineStr"/>
       <c r="K242" s="3" t="inlineStr"/>
       <c r="L242" t="inlineStr">
         <is>
-          <t>Surface Upwelling Longwave on Land-Use Tile</t>
+          <t>Roughness Length</t>
         </is>
       </c>
       <c r="M242" t="inlineStr">
         <is>
-          <t>surface_upwelling_longwave_flux_in_air</t>
+          <t>roughness_length</t>
         </is>
       </c>
       <c r="N242" t="inlineStr">
         <is>
-          <t>ACLWUPB I_ACLWUPB</t>
+          <t>ZNT</t>
         </is>
       </c>
       <c r="O242" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_rad (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
+          <t>CORDEX_Cmor: RCM_sfc_rough (lsm varset)</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>rough</t>
+          <t>rsusLut</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -16353,49 +16353,49 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>W m-2</t>
         </is>
       </c>
       <c r="E243" s="3" t="inlineStr">
         <is>
-          <t>i</t>
-        </is>
-      </c>
-      <c r="F243" s="3" t="inlineStr"/>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="F243" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G243" s="3" t="inlineStr"/>
       <c r="H243" s="3" t="inlineStr"/>
-      <c r="I243" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I243" s="3" t="inlineStr"/>
       <c r="J243" s="3" t="inlineStr"/>
       <c r="K243" s="3" t="inlineStr"/>
       <c r="L243" t="inlineStr">
         <is>
-          <t>Roughness Length</t>
+          <t>Surface Upwelling Shortwave on Land-Use Tile</t>
         </is>
       </c>
       <c r="M243" t="inlineStr">
         <is>
-          <t>roughness_length</t>
+          <t>surface_upwelling_shortwave_flux_in_air</t>
         </is>
       </c>
       <c r="N243" t="inlineStr">
         <is>
-          <t>ZNT</t>
+          <t>ACSWUPB I_ACSWUPB</t>
         </is>
       </c>
       <c r="O243" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_rough (lsm varset)</t>
+          <t>CORDEX_Cmor: RCM_sfc_rad (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>rsusLut</t>
+          <t>shrubFrac</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -16410,49 +16410,49 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>W m-2</t>
-        </is>
-      </c>
-      <c r="E244" s="3" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="F244" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E244" s="3" t="inlineStr"/>
+      <c r="F244" s="3" t="inlineStr"/>
       <c r="G244" s="3" t="inlineStr"/>
       <c r="H244" s="3" t="inlineStr"/>
-      <c r="I244" s="3" t="inlineStr"/>
+      <c r="I244" s="3" t="inlineStr">
+        <is>
+          <t>x¹</t>
+        </is>
+      </c>
       <c r="J244" s="3" t="inlineStr"/>
-      <c r="K244" s="3" t="inlineStr"/>
+      <c r="K244" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L244" t="inlineStr">
         <is>
-          <t>Surface Upwelling Shortwave on Land-Use Tile</t>
+          <t>Percentage Cover by Shrub</t>
         </is>
       </c>
       <c r="M244" t="inlineStr">
         <is>
-          <t>surface_upwelling_shortwave_flux_in_air</t>
+          <t>area_fraction</t>
         </is>
       </c>
       <c r="N244" t="inlineStr">
         <is>
-          <t>ACSWUPB I_ACSWUPB</t>
+          <t>LANDUSEF</t>
         </is>
       </c>
       <c r="O244" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_rad (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
+          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF classes grouped (landuse_field in shared_subs_v2.f90)</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>shrubFrac</t>
+          <t>sweLut</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -16467,49 +16467,49 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E245" s="3" t="inlineStr"/>
-      <c r="F245" s="3" t="inlineStr"/>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E245" s="3" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
+      </c>
+      <c r="F245" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G245" s="3" t="inlineStr"/>
       <c r="H245" s="3" t="inlineStr"/>
-      <c r="I245" s="3" t="inlineStr">
-        <is>
-          <t>x¹</t>
-        </is>
-      </c>
+      <c r="I245" s="3" t="inlineStr"/>
       <c r="J245" s="3" t="inlineStr"/>
-      <c r="K245" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K245" s="3" t="inlineStr"/>
       <c r="L245" t="inlineStr">
         <is>
-          <t>Percentage Cover by Shrub</t>
+          <t>Snow Water Equivalent on Land-Use Tile</t>
         </is>
       </c>
       <c r="M245" t="inlineStr">
         <is>
-          <t>area_fraction</t>
+          <t>lwe_thickness_of_surface_snow_amount</t>
         </is>
       </c>
       <c r="N245" t="inlineStr">
         <is>
-          <t>LANDUSEF</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="O245" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF classes grouped (landuse_field in shared_subs_v2.f90)</t>
+          <t>CORDEX_Cmor: RCM_sfc_snw (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>sweLut</t>
+          <t>tasLut</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -16524,7 +16524,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>K</t>
         </is>
       </c>
       <c r="E246" s="3" t="inlineStr">
@@ -16544,29 +16544,29 @@
       <c r="K246" s="3" t="inlineStr"/>
       <c r="L246" t="inlineStr">
         <is>
-          <t>Snow Water Equivalent on Land-Use Tile</t>
+          <t>Air temperature is the bulk temperature of the air, not the surface (skin) temperature.</t>
         </is>
       </c>
       <c r="M246" t="inlineStr">
         <is>
-          <t>lwe_thickness_of_surface_snow_amount</t>
+          <t>air_temperature</t>
         </is>
       </c>
       <c r="N246" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="O246" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_snw (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
+          <t>CORDEX_Cmor: RCM_sfc_tas (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>tasLut</t>
+          <t>tcs</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -16601,29 +16601,29 @@
       <c r="K247" s="3" t="inlineStr"/>
       <c r="L247" t="inlineStr">
         <is>
-          <t>Air temperature is the bulk temperature of the air, not the surface (skin) temperature.</t>
+          <t>Vegetation temperature, averaged over all vegetation types</t>
         </is>
       </c>
       <c r="M247" t="inlineStr">
         <is>
-          <t>air_temperature</t>
+          <t>canopy_temperature</t>
         </is>
       </c>
       <c r="N247" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>TV</t>
         </is>
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_tas (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
+          <t>CORDEX_Cmor: RCM_sfc_tcs (lsm varset)</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>tcs</t>
+          <t>tgs</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -16658,29 +16658,29 @@
       <c r="K248" s="3" t="inlineStr"/>
       <c r="L248" t="inlineStr">
         <is>
-          <t>Vegetation temperature, averaged over all vegetation types</t>
+          <t>Surface bare soil temperature</t>
         </is>
       </c>
       <c r="M248" t="inlineStr">
         <is>
-          <t>canopy_temperature</t>
+          <t>surface_temperature</t>
         </is>
       </c>
       <c r="N248" t="inlineStr">
         <is>
-          <t>TV</t>
+          <t>TGB</t>
         </is>
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_tcs (lsm varset)</t>
+          <t>CORDEX_Cmor: RCM_sfc_tgs (lsm varset)</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>tgs</t>
+          <t>tran</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -16695,12 +16695,12 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>kg m-2 s-1</t>
         </is>
       </c>
       <c r="E249" s="3" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>a</t>
         </is>
       </c>
       <c r="F249" s="3" t="inlineStr">
@@ -16715,29 +16715,29 @@
       <c r="K249" s="3" t="inlineStr"/>
       <c r="L249" t="inlineStr">
         <is>
-          <t>Surface bare soil temperature</t>
+          <t>Transpiration (may include dew formation as a negative flux).</t>
         </is>
       </c>
       <c r="M249" t="inlineStr">
         <is>
-          <t>surface_temperature</t>
+          <t>transpiration_flux</t>
         </is>
       </c>
       <c r="N249" t="inlineStr">
         <is>
-          <t>TGB</t>
+          <t>ETRAN</t>
         </is>
       </c>
       <c r="O249" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_tgs (lsm varset)</t>
+          <t>CORDEX_Cmor: RCM_sfc_tran (lsm varset)</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>tran</t>
+          <t>treeFrac</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -16752,49 +16752,49 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>kg m-2 s-1</t>
-        </is>
-      </c>
-      <c r="E250" s="3" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="F250" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E250" s="3" t="inlineStr"/>
+      <c r="F250" s="3" t="inlineStr"/>
       <c r="G250" s="3" t="inlineStr"/>
       <c r="H250" s="3" t="inlineStr"/>
-      <c r="I250" s="3" t="inlineStr"/>
+      <c r="I250" s="3" t="inlineStr">
+        <is>
+          <t>x¹</t>
+        </is>
+      </c>
       <c r="J250" s="3" t="inlineStr"/>
-      <c r="K250" s="3" t="inlineStr"/>
+      <c r="K250" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L250" t="inlineStr">
         <is>
-          <t>Transpiration (may include dew formation as a negative flux).</t>
+          <t>Tree Cover Percentage</t>
         </is>
       </c>
       <c r="M250" t="inlineStr">
         <is>
-          <t>transpiration_flux</t>
+          <t>area_fraction</t>
         </is>
       </c>
       <c r="N250" t="inlineStr">
         <is>
-          <t>ETRAN</t>
+          <t>LANDUSEF</t>
         </is>
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_tran (lsm varset)</t>
+          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF classes grouped (landuse_field in shared_subs_v2.f90)</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>treeFrac</t>
+          <t>treeFracBdlDcd</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -16829,7 +16829,7 @@
       </c>
       <c r="L251" t="inlineStr">
         <is>
-          <t>Tree Cover Percentage</t>
+          <t>This is the percentage of the entire grid cell that is covered by broadleaf deciduous trees.</t>
         </is>
       </c>
       <c r="M251" t="inlineStr">
@@ -16844,14 +16844,14 @@
       </c>
       <c r="O251" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF classes grouped (landuse_field in shared_subs_v2.f90)</t>
+          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset)</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>treeFracBdlDcd</t>
+          <t>treeFracBdlEvg</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -16886,7 +16886,7 @@
       </c>
       <c r="L252" t="inlineStr">
         <is>
-          <t>This is the percentage of the entire grid cell that is covered by broadleaf deciduous trees.</t>
+          <t>This is the percentage of the entire grid cell that is covered by broadleaf evergreen trees.</t>
         </is>
       </c>
       <c r="M252" t="inlineStr">
@@ -16908,7 +16908,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>treeFracBdlEvg</t>
+          <t>treeFracNdlDcd</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -16943,7 +16943,7 @@
       </c>
       <c r="L253" t="inlineStr">
         <is>
-          <t>This is the percentage of the entire grid cell that is covered by broadleaf evergreen trees.</t>
+          <t>This is the percentage of the entire grid cell that is covered by needleleaf deciduous trees.</t>
         </is>
       </c>
       <c r="M253" t="inlineStr">
@@ -16965,7 +16965,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>treeFracNdlDcd</t>
+          <t>tslsiLut</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -16980,49 +16980,49 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E254" s="3" t="inlineStr"/>
-      <c r="F254" s="3" t="inlineStr"/>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="E254" s="3" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
+      </c>
+      <c r="F254" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G254" s="3" t="inlineStr"/>
       <c r="H254" s="3" t="inlineStr"/>
-      <c r="I254" s="3" t="inlineStr">
-        <is>
-          <t>x¹</t>
-        </is>
-      </c>
+      <c r="I254" s="3" t="inlineStr"/>
       <c r="J254" s="3" t="inlineStr"/>
-      <c r="K254" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K254" s="3" t="inlineStr"/>
       <c r="L254" t="inlineStr">
         <is>
-          <t>This is the percentage of the entire grid cell that is covered by needleleaf deciduous trees.</t>
+          <t>Surface temperature (i.e. temperature at which long-wave radiation emitted)</t>
         </is>
       </c>
       <c r="M254" t="inlineStr">
         <is>
-          <t>area_fraction</t>
+          <t>surface_temperature</t>
         </is>
       </c>
       <c r="N254" t="inlineStr">
         <is>
-          <t>LANDUSEF</t>
+          <t>TSK</t>
         </is>
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset)</t>
+          <t>CORDEX_Cmor: RCM_sfc_ts (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>tslsiLut</t>
+          <t>urbanFrac</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -17037,49 +17037,49 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="E255" s="3" t="inlineStr">
-        <is>
-          <t>i</t>
-        </is>
-      </c>
-      <c r="F255" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E255" s="3" t="inlineStr"/>
+      <c r="F255" s="3" t="inlineStr"/>
       <c r="G255" s="3" t="inlineStr"/>
       <c r="H255" s="3" t="inlineStr"/>
-      <c r="I255" s="3" t="inlineStr"/>
+      <c r="I255" s="3" t="inlineStr">
+        <is>
+          <t>x¹</t>
+        </is>
+      </c>
       <c r="J255" s="3" t="inlineStr"/>
-      <c r="K255" s="3" t="inlineStr"/>
+      <c r="K255" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L255" t="inlineStr">
         <is>
-          <t>Surface temperature (i.e. temperature at which long-wave radiation emitted)</t>
+          <t>Urban Percentage Area Coverage</t>
         </is>
       </c>
       <c r="M255" t="inlineStr">
         <is>
-          <t>surface_temperature</t>
+          <t>area_fraction</t>
         </is>
       </c>
       <c r="N255" t="inlineStr">
         <is>
-          <t>TSK</t>
+          <t>LANDUSEF</t>
         </is>
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_sfc_ts (lut varset); no land-use tiles in WRF: the grid-cell value, with the Lut header</t>
+          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF urban classes incl. LCZ (landuse_field in shared_subs_v2.f90)</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>urbanFrac</t>
+          <t>vortmen</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -17094,106 +17094,106 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E256" s="3" t="inlineStr"/>
+          <t>s-1</t>
+        </is>
+      </c>
+      <c r="E256" s="3" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
+      </c>
       <c r="F256" s="3" t="inlineStr"/>
-      <c r="G256" s="3" t="inlineStr"/>
+      <c r="G256" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="H256" s="3" t="inlineStr"/>
-      <c r="I256" s="3" t="inlineStr">
-        <is>
-          <t>x¹</t>
-        </is>
-      </c>
+      <c r="I256" s="3" t="inlineStr"/>
       <c r="J256" s="3" t="inlineStr"/>
-      <c r="K256" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K256" s="3" t="inlineStr"/>
       <c r="L256" t="inlineStr">
         <is>
-          <t>Urban Percentage Area Coverage</t>
+          <t>relative vorticity</t>
         </is>
       </c>
       <c r="M256" t="inlineStr">
         <is>
-          <t>area_fraction</t>
+          <t>atmosphere_relative_vorticity</t>
         </is>
       </c>
       <c r="N256" t="inlineStr">
         <is>
-          <t>LANDUSEF</t>
+          <t>U V MAPFAC_U MAPFAC_V MAPFAC_M P PB</t>
         </is>
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF urban classes incl. LCZ (landuse_field in shared_subs_v2.f90)</t>
+          <t>CORDEX_Cmor: RCM_plev_vortmen (plev_vortmen0/1 varsets), as vortmen&lt;p&gt; on each pressure level (1000 to 30 hPa); m^2 [d(v/m_v)/dx - d(u/m_u)/dy] as wrf-python; every wp_step hours (grid ini)</t>
         </is>
       </c>
     </row>
     <row r="257">
-      <c r="A257" s="4" t="inlineStr">
-        <is>
-          <t>vortmen</t>
-        </is>
-      </c>
-      <c r="B257" s="4" t="inlineStr">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>wap</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
         <is>
           <t>FPS-LUCAS</t>
         </is>
       </c>
-      <c r="C257" s="4" t="inlineStr">
+      <c r="C257" t="inlineStr">
         <is>
           <t>TIER 1</t>
         </is>
       </c>
-      <c r="D257" s="4" t="inlineStr">
-        <is>
-          <t>s-1</t>
-        </is>
-      </c>
-      <c r="E257" s="5" t="inlineStr">
-        <is>
-          <t>i</t>
-        </is>
-      </c>
-      <c r="F257" s="5" t="inlineStr"/>
-      <c r="G257" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="H257" s="5" t="inlineStr"/>
-      <c r="I257" s="5" t="inlineStr"/>
-      <c r="J257" s="5" t="inlineStr"/>
-      <c r="K257" s="5" t="inlineStr"/>
-      <c r="L257" s="4" t="inlineStr">
-        <is>
-          <t>relative vorticity</t>
-        </is>
-      </c>
-      <c r="M257" s="4" t="inlineStr">
-        <is>
-          <t>atmosphere_relative_vorticity</t>
-        </is>
-      </c>
-      <c r="N257" s="4" t="inlineStr">
-        <is>
-          <t>U V MAPFAC_U MAPFAC_V MAPFAC_M P PB</t>
-        </is>
-      </c>
-      <c r="O257" s="4" t="inlineStr">
-        <is>
-          <t>not produced by CORDEX_Cmor; header ready; relative vorticity on pressure levels</t>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Pa s-1</t>
+        </is>
+      </c>
+      <c r="E257" s="3" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
+      </c>
+      <c r="F257" s="3" t="inlineStr"/>
+      <c r="G257" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H257" s="3" t="inlineStr"/>
+      <c r="I257" s="3" t="inlineStr"/>
+      <c r="J257" s="3" t="inlineStr"/>
+      <c r="K257" s="3" t="inlineStr"/>
+      <c r="L257" t="inlineStr">
+        <is>
+          <t>omega</t>
+        </is>
+      </c>
+      <c r="M257" t="inlineStr">
+        <is>
+          <t>lagrangian_tendency_of_air_pressure</t>
+        </is>
+      </c>
+      <c r="N257" t="inlineStr">
+        <is>
+          <t>W T QVAPOR P PB</t>
+        </is>
+      </c>
+      <c r="O257" t="inlineStr">
+        <is>
+          <t>CORDEX_Cmor: RCM_plev_wap (plev_wap varset), as wap&lt;p&gt; on each pressure level (1000 to 30 hPa); omega = -rho g w; every wp_step hours (grid ini)</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>wap</t>
+          <t>slthick</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -17208,49 +17208,49 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>Pa s-1</t>
-        </is>
-      </c>
-      <c r="E258" s="3" t="inlineStr">
-        <is>
-          <t>i</t>
-        </is>
-      </c>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E258" s="3" t="inlineStr"/>
       <c r="F258" s="3" t="inlineStr"/>
-      <c r="G258" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="G258" s="3" t="inlineStr"/>
       <c r="H258" s="3" t="inlineStr"/>
-      <c r="I258" s="3" t="inlineStr"/>
+      <c r="I258" s="3" t="inlineStr">
+        <is>
+          <t>x¹</t>
+        </is>
+      </c>
       <c r="J258" s="3" t="inlineStr"/>
-      <c r="K258" s="3" t="inlineStr"/>
+      <c r="K258" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L258" t="inlineStr">
         <is>
-          <t>omega</t>
+          <t>Thickness of Soil Layers</t>
         </is>
       </c>
       <c r="M258" t="inlineStr">
         <is>
-          <t>lagrangian_tendency_of_air_pressure</t>
+          <t>cell_thickness</t>
         </is>
       </c>
       <c r="N258" t="inlineStr">
         <is>
-          <t>W T QVAPOR P PB</t>
+          <t>DZS</t>
         </is>
       </c>
       <c r="O258" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_plev_wap (plev_wap varset), as wap&lt;p&gt; on each pressure level (1000 to 30 hPa); omega = -rho g w; every wp_step hours (grid ini)</t>
+          <t>CORDEX_Cmor: RCM_fx_slthick (fx varset)</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>slthick</t>
+          <t>lcvr</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -17258,18 +17258,18 @@
           <t>FPS-LUCAS</t>
         </is>
       </c>
-      <c r="C259" t="inlineStr">
-        <is>
-          <t>TIER 1</t>
-        </is>
-      </c>
+      <c r="C259" t="inlineStr"/>
       <c r="D259" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E259" s="3" t="inlineStr"/>
-      <c r="F259" s="3" t="inlineStr"/>
+      <c r="F259" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G259" s="3" t="inlineStr"/>
       <c r="H259" s="3" t="inlineStr"/>
       <c r="I259" s="3" t="inlineStr">
@@ -17285,88 +17285,31 @@
       </c>
       <c r="L259" t="inlineStr">
         <is>
-          <t>Thickness of Soil Layers</t>
-        </is>
-      </c>
-      <c r="M259" t="inlineStr">
-        <is>
-          <t>cell_thickness</t>
-        </is>
-      </c>
+          <t>Land Cover Dominant Class</t>
+        </is>
+      </c>
+      <c r="M259" t="inlineStr"/>
       <c r="N259" t="inlineStr">
         <is>
-          <t>DZS</t>
+          <t>LU_INDEX</t>
         </is>
       </c>
       <c r="O259" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_fx_slthick (fx varset)</t>
-        </is>
-      </c>
-    </row>
-    <row r="260">
-      <c r="A260" t="inlineStr">
-        <is>
-          <t>lcvr</t>
-        </is>
-      </c>
-      <c r="B260" t="inlineStr">
-        <is>
-          <t>FPS-LUCAS</t>
-        </is>
-      </c>
-      <c r="C260" t="inlineStr"/>
-      <c r="D260" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E260" s="3" t="inlineStr"/>
-      <c r="F260" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="G260" s="3" t="inlineStr"/>
-      <c r="H260" s="3" t="inlineStr"/>
-      <c r="I260" s="3" t="inlineStr">
-        <is>
-          <t>x¹</t>
-        </is>
-      </c>
-      <c r="J260" s="3" t="inlineStr"/>
-      <c r="K260" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="L260" t="inlineStr">
-        <is>
-          <t>Land Cover Dominant Class</t>
-        </is>
-      </c>
-      <c r="M260" t="inlineStr"/>
-      <c r="N260" t="inlineStr">
-        <is>
-          <t>LU_INDEX</t>
-        </is>
-      </c>
-      <c r="O260" t="inlineStr">
-        <is>
           <t>CORDEX_Cmor: RCM_fx_lcvr (fx varset, from geo_em) and RCM_sfc_landuse (landuse varset); LU_INDEX (dominant land-use class); hourly from wrfout; not in the phase 2 workbook list</t>
         </is>
       </c>
     </row>
-    <row r="261"/>
-    <row r="262">
-      <c r="A262" s="6" t="inlineStr">
+    <row r="260"/>
+    <row r="261">
+      <c r="A261" s="6" t="inlineStr">
         <is>
           <t>¹ LUCAS frequency: requested by FPS-LUCAS but not by CORDEX-CMIP6 for this variable; time-invariant (fx) variables are assumed to be also daily variables in LUCAS</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O260"/>
+  <autoFilter ref="A1:O259"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
albc: canopy albedo from ALBEDO and the vegetated fraction (LANDUSEF)
- RCM_sfc_albc (lsm varset, 1hr instantaneous): albc = cnc/100 x ALBEDO, cnc the
  vegetated % of the cell (tree + shrub + grass + crop classes of LANDUSEF, as cnc in
  landuse_field) from the same wrfout file; sea missing; rounded to 1e-4.
- landuse_field: albc uses the cnc weights.
- header_albc: wrfvar ALBEDO, time: point; aggregation row (day, mon mean);
  README and variable list updated; lsm TIME 16 h.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QusijEwmX4bwsbKvYikBaV
</commit_message>
<xml_diff>
--- a/CORDEX_Cmor_variables.xlsx
+++ b/CORDEX_Cmor_variables.xlsx
@@ -15025,59 +15025,59 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="4" t="inlineStr">
+      <c r="A220" t="inlineStr">
         <is>
           <t>albc</t>
         </is>
       </c>
-      <c r="B220" s="4" t="inlineStr">
+      <c r="B220" t="inlineStr">
         <is>
           <t>FPS-LUCAS</t>
         </is>
       </c>
-      <c r="C220" s="4" t="inlineStr">
+      <c r="C220" t="inlineStr">
         <is>
           <t>TIER 1</t>
         </is>
       </c>
-      <c r="D220" s="4" t="inlineStr">
+      <c r="D220" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E220" s="5" t="inlineStr">
-        <is>
-          <t>i</t>
-        </is>
-      </c>
-      <c r="F220" s="5" t="inlineStr"/>
-      <c r="G220" s="5" t="inlineStr"/>
-      <c r="H220" s="5" t="inlineStr"/>
-      <c r="I220" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="J220" s="5" t="inlineStr"/>
-      <c r="K220" s="5" t="inlineStr"/>
-      <c r="L220" s="4" t="inlineStr">
+      <c r="E220" s="3" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
+      </c>
+      <c r="F220" s="3" t="inlineStr"/>
+      <c r="G220" s="3" t="inlineStr"/>
+      <c r="H220" s="3" t="inlineStr"/>
+      <c r="I220" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J220" s="3" t="inlineStr"/>
+      <c r="K220" s="3" t="inlineStr"/>
+      <c r="L220" t="inlineStr">
         <is>
           <t>Albedo of the vegetation: fraction of incoming solar radiation which is reflected before reaching the ground.</t>
         </is>
       </c>
-      <c r="M220" s="4" t="inlineStr">
+      <c r="M220" t="inlineStr">
         <is>
           <t>canopy_albedo</t>
         </is>
       </c>
-      <c r="N220" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O220" s="4" t="inlineStr">
-        <is>
-          <t>not produced by CORDEX_Cmor; header ready; no canopy albedo in the WRF output</t>
+      <c r="N220" t="inlineStr">
+        <is>
+          <t>ALBEDO LANDUSEF</t>
+        </is>
+      </c>
+      <c r="O220" t="inlineStr">
+        <is>
+          <t>CORDEX_Cmor: RCM_sfc_albc (lsm varset); ALBEDO x vegetated fraction of the cell (LANDUSEF classes of cnc)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
pastureFrac from the grassland land-use class
- landuse_field: pastureFrac = 100 LANDUSEF of the grassland class (MODIS 10,
  USGS 7); the WRF tables have no pasture class. It is also part of grassFrac.
- varsets (all three): pastureFrac in fx (RCM_fx_landuse) and landuse
  (RCM_sfc_landuse); header, aggregation row, README and variable list updated.
- All FPS-LUCAS variables are now produced (hu left out on request).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QusijEwmX4bwsbKvYikBaV
</commit_message>
<xml_diff>
--- a/CORDEX_Cmor_variables.xlsx
+++ b/CORDEX_Cmor_variables.xlsx
@@ -16108,59 +16108,59 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="4" t="inlineStr">
+      <c r="A239" t="inlineStr">
         <is>
           <t>pastureFrac</t>
         </is>
       </c>
-      <c r="B239" s="4" t="inlineStr">
+      <c r="B239" t="inlineStr">
         <is>
           <t>FPS-LUCAS</t>
         </is>
       </c>
-      <c r="C239" s="4" t="inlineStr">
+      <c r="C239" t="inlineStr">
         <is>
           <t>TIER 1</t>
         </is>
       </c>
-      <c r="D239" s="4" t="inlineStr">
+      <c r="D239" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E239" s="5" t="inlineStr"/>
-      <c r="F239" s="5" t="inlineStr"/>
-      <c r="G239" s="5" t="inlineStr"/>
-      <c r="H239" s="5" t="inlineStr"/>
-      <c r="I239" s="5" t="inlineStr">
+      <c r="E239" s="3" t="inlineStr"/>
+      <c r="F239" s="3" t="inlineStr"/>
+      <c r="G239" s="3" t="inlineStr"/>
+      <c r="H239" s="3" t="inlineStr"/>
+      <c r="I239" s="3" t="inlineStr">
         <is>
           <t>x¹</t>
         </is>
       </c>
-      <c r="J239" s="5" t="inlineStr"/>
-      <c r="K239" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="L239" s="4" t="inlineStr">
+      <c r="J239" s="3" t="inlineStr"/>
+      <c r="K239" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="L239" t="inlineStr">
         <is>
           <t>Percentage of Land Which Is Anthropogenic Pasture</t>
         </is>
       </c>
-      <c r="M239" s="4" t="inlineStr">
+      <c r="M239" t="inlineStr">
         <is>
           <t>area_fraction</t>
         </is>
       </c>
-      <c r="N239" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O239" s="4" t="inlineStr">
-        <is>
-          <t>not produced by CORDEX_Cmor; header ready; no pasture class in the WRF land-use tables</t>
+      <c r="N239" t="inlineStr">
+        <is>
+          <t>LANDUSEF</t>
+        </is>
+      </c>
+      <c r="O239" t="inlineStr">
+        <is>
+          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Variable list: project CORDEX-CMIP6 for the variables shared with FPS-LUCAS
- The 60 variables requested by both CORDEX-CMIP6 and FPS-LUCAS now have project
  "CORDEX-CMIP6" (was "CORDEX-CMIP6, FPS-LUCAS"); the LUCAS-only frequencies keep
  their x¹ and the legend, and Priority keeps the LUCAS priority.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QusijEwmX4bwsbKvYikBaV
</commit_message>
<xml_diff>
--- a/CORDEX_Cmor_variables.xlsx
+++ b/CORDEX_Cmor_variables.xlsx
@@ -546,7 +546,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -668,7 +668,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -855,7 +855,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -985,7 +985,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1245,7 +1245,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1310,7 +1310,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1871,7 +1871,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2200,7 +2200,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2468,7 +2468,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2712,7 +2712,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2972,7 +2972,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -3297,7 +3297,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -3431,7 +3431,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3569,7 +3569,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3638,7 +3638,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -3898,7 +3898,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -3963,7 +3963,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -4296,7 +4296,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -4507,7 +4507,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -4718,7 +4718,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -5209,7 +5209,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -5700,7 +5700,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -5907,7 +5907,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -6601,7 +6601,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -6881,7 +6881,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -7092,7 +7092,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -7303,7 +7303,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -7794,7 +7794,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -8005,7 +8005,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -8216,7 +8216,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -8878,7 +8878,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -9646,7 +9646,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -9776,7 +9776,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -13572,7 +13572,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -13625,7 +13625,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -13894,7 +13894,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>CORDEX-CMIP6, FPS-LUCAS</t>
+          <t>CORDEX-CMIP6</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">

</xml_diff>

<commit_message>
Variable list: LUCAS priority only where it differs from the CORDEX one
19 shared variables had the same priority in both lists (e.g. "CORE; LUCAS CORE");
they now show only the CORDEX priority. The 41 with a different LUCAS priority keep
it (e.g. "TIER 1; LUCAS CORE").

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QusijEwmX4bwsbKvYikBaV
</commit_message>
<xml_diff>
--- a/CORDEX_Cmor_variables.xlsx
+++ b/CORDEX_Cmor_variables.xlsx
@@ -551,7 +551,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CORE; LUCAS CORE</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CORE; LUCAS CORE</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -673,7 +673,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CORE; LUCAS CORE</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CORE; LUCAS CORE</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CORE; LUCAS CORE</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CORE; LUCAS CORE</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CORE; LUCAS CORE</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CORE; LUCAS CORE</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CORE; LUCAS CORE</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CORE; LUCAS CORE</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CORE; LUCAS CORE</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CORE; LUCAS CORE</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CORE; LUCAS CORE</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1380,7 +1380,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CORE; LUCAS CORE</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CORE; LUCAS CORE</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CORE; LUCAS CORE</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CORE; LUCAS CORE</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1876,7 +1876,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>TIER 1; LUCAS TIER 1</t>
+          <t>TIER 1</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2071,7 +2071,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>TIER 1; LUCAS TIER 1</t>
+          <t>TIER 1</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">

</xml_diff>

<commit_message>
Variable tables: landuse_field is in landuse_subs.f90
The comment column of CORDEX_Cmor_variables.csv and .xlsx (7 land-use
fractions) still named shared_subs_v2.f90. The xlsx is edited in its
shared strings only, so its formatting is kept.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QusijEwmX4bwsbKvYikBaV
</commit_message>
<xml_diff>
--- a/CORDEX_Cmor_variables.xlsx
+++ b/CORDEX_Cmor_variables.xlsx
@@ -15106,7 +15106,7 @@
       </c>
       <c r="O221" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF classes grouped (landuse_field in shared_subs_v2.f90)</t>
+          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF classes grouped (landuse_field in landuse_subs.f90)</t>
         </is>
       </c>
     </row>
@@ -15163,7 +15163,7 @@
       </c>
       <c r="O222" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF tree+shrub+grass+crop (landuse_field in shared_subs_v2.f90)</t>
+          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF tree+shrub+grass+crop (landuse_field in landuse_subs.f90)</t>
         </is>
       </c>
     </row>
@@ -15220,7 +15220,7 @@
       </c>
       <c r="O223" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF classes grouped (landuse_field in shared_subs_v2.f90)</t>
+          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF classes grouped (landuse_field in landuse_subs.f90)</t>
         </is>
       </c>
     </row>
@@ -15448,7 +15448,7 @@
       </c>
       <c r="O227" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF classes grouped (landuse_field in shared_subs_v2.f90)</t>
+          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF classes grouped (landuse_field in landuse_subs.f90)</t>
         </is>
       </c>
     </row>
@@ -16417,7 +16417,7 @@
       </c>
       <c r="O244" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF classes grouped (landuse_field in shared_subs_v2.f90)</t>
+          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF classes grouped (landuse_field in landuse_subs.f90)</t>
         </is>
       </c>
     </row>
@@ -16759,7 +16759,7 @@
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF classes grouped (landuse_field in shared_subs_v2.f90)</t>
+          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF classes grouped (landuse_field in landuse_subs.f90)</t>
         </is>
       </c>
     </row>
@@ -17044,7 +17044,7 @@
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF urban classes incl. LCZ (landuse_field in shared_subs_v2.f90)</t>
+          <t>CORDEX_Cmor: RCM_fx_landuse (fx varset) and RCM_sfc_landuse (landuse varset); LANDUSEF urban classes incl. LCZ (landuse_field in landuse_subs.f90)</t>
         </is>
       </c>
     </row>

</xml_diff>